<commit_message>
Data up to 18-OCT-2026
</commit_message>
<xml_diff>
--- a/data/dashboard-data.xlsx
+++ b/data/dashboard-data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28815" windowHeight="13980" tabRatio="488"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28815" windowHeight="13980" tabRatio="488" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="DAILY_ENTRY" sheetId="2" r:id="rId1"/>
@@ -892,6 +892,59 @@
     <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -915,59 +968,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1239,56 +1239,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="30" customHeight="1">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="63" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="58" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="57" t="s">
+      <c r="B1" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="62" t="s">
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="67" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="57" t="s">
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="62" t="s">
         <v>3</v>
       </c>
-      <c r="J1" s="57"/>
-      <c r="K1" s="57"/>
-      <c r="L1" s="62" t="s">
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="67" t="s">
         <v>4</v>
       </c>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="57" t="s">
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="62" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="57"/>
-      <c r="Q1" s="57"/>
-      <c r="R1" s="57" t="s">
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62" t="s">
         <v>6</v>
       </c>
-      <c r="S1" s="57"/>
-      <c r="T1" s="57"/>
-      <c r="U1" s="63" t="s">
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="59" t="s">
         <v>7</v>
       </c>
-      <c r="V1" s="64"/>
-      <c r="W1" s="64"/>
-      <c r="X1" s="64"/>
-      <c r="Y1" s="64"/>
-      <c r="Z1" s="64"/>
-      <c r="AA1" s="64"/>
-      <c r="AB1" s="65"/>
+      <c r="V1" s="60"/>
+      <c r="W1" s="60"/>
+      <c r="X1" s="60"/>
+      <c r="Y1" s="60"/>
+      <c r="Z1" s="60"/>
+      <c r="AA1" s="60"/>
+      <c r="AB1" s="61"/>
     </row>
     <row r="2" spans="1:28" ht="60.75" customHeight="1">
-      <c r="A2" s="58"/>
-      <c r="B2" s="58"/>
+      <c r="A2" s="63"/>
+      <c r="B2" s="63"/>
       <c r="C2" s="2" t="s">
         <v>8</v>
       </c>
@@ -1369,7 +1369,7 @@
       </c>
     </row>
     <row r="3" spans="1:28" ht="15.75" thickBot="1">
-      <c r="A3" s="59" t="s">
+      <c r="A3" s="64" t="s">
         <v>29</v>
       </c>
       <c r="B3" s="3">
@@ -1442,7 +1442,7 @@
       </c>
     </row>
     <row r="4" spans="1:28">
-      <c r="A4" s="60"/>
+      <c r="A4" s="65"/>
       <c r="B4" s="3">
         <v>46114</v>
       </c>
@@ -1511,7 +1511,7 @@
       <c r="AB4" s="4"/>
     </row>
     <row r="5" spans="1:28">
-      <c r="A5" s="60"/>
+      <c r="A5" s="65"/>
       <c r="B5" s="3">
         <v>46115</v>
       </c>
@@ -1578,7 +1578,7 @@
       <c r="AB5" s="4"/>
     </row>
     <row r="6" spans="1:28">
-      <c r="A6" s="60"/>
+      <c r="A6" s="65"/>
       <c r="B6" s="3">
         <v>46116</v>
       </c>
@@ -1645,7 +1645,7 @@
       <c r="AB6" s="4"/>
     </row>
     <row r="7" spans="1:28">
-      <c r="A7" s="60"/>
+      <c r="A7" s="65"/>
       <c r="B7" s="3">
         <v>46117</v>
       </c>
@@ -1712,7 +1712,7 @@
       <c r="AB7" s="4"/>
     </row>
     <row r="8" spans="1:28">
-      <c r="A8" s="60"/>
+      <c r="A8" s="65"/>
       <c r="B8" s="3">
         <v>46118</v>
       </c>
@@ -1779,7 +1779,7 @@
       <c r="AB8" s="4"/>
     </row>
     <row r="9" spans="1:28">
-      <c r="A9" s="60"/>
+      <c r="A9" s="65"/>
       <c r="B9" s="3">
         <v>46119</v>
       </c>
@@ -1846,7 +1846,7 @@
       <c r="AB9" s="4"/>
     </row>
     <row r="10" spans="1:28">
-      <c r="A10" s="60"/>
+      <c r="A10" s="65"/>
       <c r="B10" s="3">
         <v>46120</v>
       </c>
@@ -1913,7 +1913,7 @@
       <c r="AB10" s="4"/>
     </row>
     <row r="11" spans="1:28">
-      <c r="A11" s="60"/>
+      <c r="A11" s="65"/>
       <c r="B11" s="3">
         <v>46121</v>
       </c>
@@ -1980,7 +1980,7 @@
       <c r="AB11" s="4"/>
     </row>
     <row r="12" spans="1:28">
-      <c r="A12" s="60"/>
+      <c r="A12" s="65"/>
       <c r="B12" s="3">
         <v>46122</v>
       </c>
@@ -2047,7 +2047,7 @@
       <c r="AB12" s="4"/>
     </row>
     <row r="13" spans="1:28">
-      <c r="A13" s="60"/>
+      <c r="A13" s="65"/>
       <c r="B13" s="3">
         <v>46123</v>
       </c>
@@ -2114,7 +2114,7 @@
       <c r="AB13" s="4"/>
     </row>
     <row r="14" spans="1:28">
-      <c r="A14" s="60"/>
+      <c r="A14" s="65"/>
       <c r="B14" s="3">
         <v>46124</v>
       </c>
@@ -2181,7 +2181,7 @@
       <c r="AB14" s="4"/>
     </row>
     <row r="15" spans="1:28">
-      <c r="A15" s="60"/>
+      <c r="A15" s="65"/>
       <c r="B15" s="3">
         <v>46125</v>
       </c>
@@ -2248,7 +2248,7 @@
       <c r="AB15" s="4"/>
     </row>
     <row r="16" spans="1:28">
-      <c r="A16" s="60"/>
+      <c r="A16" s="65"/>
       <c r="B16" s="3">
         <v>46126</v>
       </c>
@@ -2315,7 +2315,7 @@
       <c r="AB16" s="4"/>
     </row>
     <row r="17" spans="1:28">
-      <c r="A17" s="60"/>
+      <c r="A17" s="65"/>
       <c r="B17" s="3">
         <v>46127</v>
       </c>
@@ -2382,7 +2382,7 @@
       <c r="AB17" s="4"/>
     </row>
     <row r="18" spans="1:28">
-      <c r="A18" s="60"/>
+      <c r="A18" s="65"/>
       <c r="B18" s="3">
         <v>46128</v>
       </c>
@@ -2449,7 +2449,7 @@
       <c r="AB18" s="4"/>
     </row>
     <row r="19" spans="1:28">
-      <c r="A19" s="60"/>
+      <c r="A19" s="65"/>
       <c r="B19" s="3">
         <v>46129</v>
       </c>
@@ -2516,7 +2516,7 @@
       <c r="AB19" s="4"/>
     </row>
     <row r="20" spans="1:28">
-      <c r="A20" s="60"/>
+      <c r="A20" s="65"/>
       <c r="B20" s="3">
         <v>46130</v>
       </c>
@@ -2583,7 +2583,7 @@
       <c r="AB20" s="4"/>
     </row>
     <row r="21" spans="1:28">
-      <c r="A21" s="60"/>
+      <c r="A21" s="65"/>
       <c r="B21" s="3">
         <v>46131</v>
       </c>
@@ -2650,7 +2650,7 @@
       <c r="AB21" s="4"/>
     </row>
     <row r="22" spans="1:28">
-      <c r="A22" s="60"/>
+      <c r="A22" s="65"/>
       <c r="B22" s="3">
         <v>46132</v>
       </c>
@@ -2717,7 +2717,7 @@
       <c r="AB22" s="4"/>
     </row>
     <row r="23" spans="1:28">
-      <c r="A23" s="60"/>
+      <c r="A23" s="65"/>
       <c r="B23" s="3">
         <v>46133</v>
       </c>
@@ -2784,7 +2784,7 @@
       <c r="AB23" s="4"/>
     </row>
     <row r="24" spans="1:28">
-      <c r="A24" s="60"/>
+      <c r="A24" s="65"/>
       <c r="B24" s="3">
         <v>46134</v>
       </c>
@@ -2851,7 +2851,7 @@
       <c r="AB24" s="4"/>
     </row>
     <row r="25" spans="1:28">
-      <c r="A25" s="60"/>
+      <c r="A25" s="65"/>
       <c r="B25" s="3">
         <v>46135</v>
       </c>
@@ -2918,7 +2918,7 @@
       <c r="AB25" s="4"/>
     </row>
     <row r="26" spans="1:28">
-      <c r="A26" s="60"/>
+      <c r="A26" s="65"/>
       <c r="B26" s="3">
         <v>46136</v>
       </c>
@@ -2985,7 +2985,7 @@
       <c r="AB26" s="4"/>
     </row>
     <row r="27" spans="1:28">
-      <c r="A27" s="60"/>
+      <c r="A27" s="65"/>
       <c r="B27" s="3">
         <v>46137</v>
       </c>
@@ -3052,7 +3052,7 @@
       <c r="AB27" s="4"/>
     </row>
     <row r="28" spans="1:28">
-      <c r="A28" s="60"/>
+      <c r="A28" s="65"/>
       <c r="B28" s="3">
         <v>46138</v>
       </c>
@@ -3119,7 +3119,7 @@
       <c r="AB28" s="4"/>
     </row>
     <row r="29" spans="1:28">
-      <c r="A29" s="60"/>
+      <c r="A29" s="65"/>
       <c r="B29" s="3">
         <v>46139</v>
       </c>
@@ -3186,7 +3186,7 @@
       <c r="AB29" s="4"/>
     </row>
     <row r="30" spans="1:28">
-      <c r="A30" s="60"/>
+      <c r="A30" s="65"/>
       <c r="B30" s="3">
         <v>46140</v>
       </c>
@@ -3253,7 +3253,7 @@
       <c r="AB30" s="4"/>
     </row>
     <row r="31" spans="1:28">
-      <c r="A31" s="60"/>
+      <c r="A31" s="65"/>
       <c r="B31" s="3">
         <v>46141</v>
       </c>
@@ -3320,7 +3320,7 @@
       <c r="AB31" s="4"/>
     </row>
     <row r="32" spans="1:28" ht="15.75" thickBot="1">
-      <c r="A32" s="61"/>
+      <c r="A32" s="66"/>
       <c r="B32" s="3">
         <v>46142</v>
       </c>
@@ -3387,7 +3387,7 @@
       <c r="AB32" s="4"/>
     </row>
     <row r="33" spans="1:28" ht="15.75" customHeight="1">
-      <c r="A33" s="55" t="s">
+      <c r="A33" s="74" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="7">
@@ -3456,7 +3456,7 @@
       <c r="AB33" s="8"/>
     </row>
     <row r="34" spans="1:28">
-      <c r="A34" s="53"/>
+      <c r="A34" s="72"/>
       <c r="B34" s="3">
         <v>46144</v>
       </c>
@@ -3523,7 +3523,7 @@
       <c r="AB34" s="4"/>
     </row>
     <row r="35" spans="1:28">
-      <c r="A35" s="53"/>
+      <c r="A35" s="72"/>
       <c r="B35" s="3">
         <v>46145</v>
       </c>
@@ -3590,7 +3590,7 @@
       <c r="AB35" s="4"/>
     </row>
     <row r="36" spans="1:28">
-      <c r="A36" s="53"/>
+      <c r="A36" s="72"/>
       <c r="B36" s="3">
         <v>46146</v>
       </c>
@@ -3659,7 +3659,7 @@
       <c r="AB36" s="4"/>
     </row>
     <row r="37" spans="1:28">
-      <c r="A37" s="53"/>
+      <c r="A37" s="72"/>
       <c r="B37" s="3">
         <v>46147</v>
       </c>
@@ -3728,7 +3728,7 @@
       <c r="AB37" s="4"/>
     </row>
     <row r="38" spans="1:28">
-      <c r="A38" s="53"/>
+      <c r="A38" s="72"/>
       <c r="B38" s="3">
         <v>46148</v>
       </c>
@@ -3797,7 +3797,7 @@
       <c r="AB38" s="4"/>
     </row>
     <row r="39" spans="1:28">
-      <c r="A39" s="53"/>
+      <c r="A39" s="72"/>
       <c r="B39" s="3">
         <v>46149</v>
       </c>
@@ -3866,7 +3866,7 @@
       <c r="AB39" s="4"/>
     </row>
     <row r="40" spans="1:28">
-      <c r="A40" s="53"/>
+      <c r="A40" s="72"/>
       <c r="B40" s="3">
         <v>46150</v>
       </c>
@@ -3935,7 +3935,7 @@
       <c r="AB40" s="4"/>
     </row>
     <row r="41" spans="1:28">
-      <c r="A41" s="53"/>
+      <c r="A41" s="72"/>
       <c r="B41" s="3">
         <v>46151</v>
       </c>
@@ -4004,7 +4004,7 @@
       <c r="AB41" s="4"/>
     </row>
     <row r="42" spans="1:28">
-      <c r="A42" s="53"/>
+      <c r="A42" s="72"/>
       <c r="B42" s="3">
         <v>46152</v>
       </c>
@@ -4073,7 +4073,7 @@
       <c r="AB42" s="4"/>
     </row>
     <row r="43" spans="1:28">
-      <c r="A43" s="53"/>
+      <c r="A43" s="72"/>
       <c r="B43" s="3">
         <v>46153</v>
       </c>
@@ -4142,7 +4142,7 @@
       <c r="AB43" s="4"/>
     </row>
     <row r="44" spans="1:28">
-      <c r="A44" s="53"/>
+      <c r="A44" s="72"/>
       <c r="B44" s="3">
         <v>46154</v>
       </c>
@@ -4211,7 +4211,7 @@
       <c r="AB44" s="4"/>
     </row>
     <row r="45" spans="1:28">
-      <c r="A45" s="53"/>
+      <c r="A45" s="72"/>
       <c r="B45" s="3">
         <v>46155</v>
       </c>
@@ -4280,7 +4280,7 @@
       <c r="AB45" s="4"/>
     </row>
     <row r="46" spans="1:28">
-      <c r="A46" s="53"/>
+      <c r="A46" s="72"/>
       <c r="B46" s="3">
         <v>46156</v>
       </c>
@@ -4349,7 +4349,7 @@
       <c r="AB46" s="4"/>
     </row>
     <row r="47" spans="1:28">
-      <c r="A47" s="53"/>
+      <c r="A47" s="72"/>
       <c r="B47" s="3">
         <v>46157</v>
       </c>
@@ -4418,7 +4418,7 @@
       <c r="AB47" s="4"/>
     </row>
     <row r="48" spans="1:28">
-      <c r="A48" s="53"/>
+      <c r="A48" s="72"/>
       <c r="B48" s="3">
         <v>46158</v>
       </c>
@@ -4487,7 +4487,7 @@
       <c r="AB48" s="4"/>
     </row>
     <row r="49" spans="1:28">
-      <c r="A49" s="53"/>
+      <c r="A49" s="72"/>
       <c r="B49" s="3">
         <v>46159</v>
       </c>
@@ -4556,7 +4556,7 @@
       <c r="AB49" s="4"/>
     </row>
     <row r="50" spans="1:28">
-      <c r="A50" s="53"/>
+      <c r="A50" s="72"/>
       <c r="B50" s="3">
         <v>46160</v>
       </c>
@@ -4625,7 +4625,7 @@
       <c r="AB50" s="4"/>
     </row>
     <row r="51" spans="1:28">
-      <c r="A51" s="53"/>
+      <c r="A51" s="72"/>
       <c r="B51" s="3">
         <v>46161</v>
       </c>
@@ -4694,7 +4694,7 @@
       <c r="AB51" s="4"/>
     </row>
     <row r="52" spans="1:28">
-      <c r="A52" s="53"/>
+      <c r="A52" s="72"/>
       <c r="B52" s="3">
         <v>46162</v>
       </c>
@@ -4763,7 +4763,7 @@
       <c r="AB52" s="4"/>
     </row>
     <row r="53" spans="1:28">
-      <c r="A53" s="53"/>
+      <c r="A53" s="72"/>
       <c r="B53" s="3">
         <v>46163</v>
       </c>
@@ -4832,7 +4832,7 @@
       <c r="AB53" s="4"/>
     </row>
     <row r="54" spans="1:28">
-      <c r="A54" s="53"/>
+      <c r="A54" s="72"/>
       <c r="B54" s="3">
         <v>46164</v>
       </c>
@@ -4901,7 +4901,7 @@
       <c r="AB54" s="4"/>
     </row>
     <row r="55" spans="1:28">
-      <c r="A55" s="53"/>
+      <c r="A55" s="72"/>
       <c r="B55" s="3">
         <v>46165</v>
       </c>
@@ -4970,7 +4970,7 @@
       <c r="AB55" s="4"/>
     </row>
     <row r="56" spans="1:28">
-      <c r="A56" s="53"/>
+      <c r="A56" s="72"/>
       <c r="B56" s="3">
         <v>46166</v>
       </c>
@@ -5041,7 +5041,7 @@
       </c>
     </row>
     <row r="57" spans="1:28">
-      <c r="A57" s="53"/>
+      <c r="A57" s="72"/>
       <c r="B57" s="3">
         <v>46167</v>
       </c>
@@ -5112,7 +5112,7 @@
       </c>
     </row>
     <row r="58" spans="1:28">
-      <c r="A58" s="53"/>
+      <c r="A58" s="72"/>
       <c r="B58" s="3">
         <v>46168</v>
       </c>
@@ -5183,7 +5183,7 @@
       </c>
     </row>
     <row r="59" spans="1:28">
-      <c r="A59" s="53"/>
+      <c r="A59" s="72"/>
       <c r="B59" s="3">
         <v>46169</v>
       </c>
@@ -5254,7 +5254,7 @@
       </c>
     </row>
     <row r="60" spans="1:28">
-      <c r="A60" s="53"/>
+      <c r="A60" s="72"/>
       <c r="B60" s="3">
         <v>46170</v>
       </c>
@@ -5325,7 +5325,7 @@
       </c>
     </row>
     <row r="61" spans="1:28">
-      <c r="A61" s="53"/>
+      <c r="A61" s="72"/>
       <c r="B61" s="3">
         <v>46171</v>
       </c>
@@ -5396,7 +5396,7 @@
       </c>
     </row>
     <row r="62" spans="1:28">
-      <c r="A62" s="53"/>
+      <c r="A62" s="72"/>
       <c r="B62" s="3">
         <v>46172</v>
       </c>
@@ -5467,7 +5467,7 @@
       </c>
     </row>
     <row r="63" spans="1:28" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A63" s="56"/>
+      <c r="A63" s="75"/>
       <c r="B63" s="3">
         <v>46173</v>
       </c>
@@ -5538,7 +5538,7 @@
       </c>
     </row>
     <row r="64" spans="1:28" ht="25.5" customHeight="1">
-      <c r="A64" s="49" t="s">
+      <c r="A64" s="68" t="s">
         <v>31</v>
       </c>
       <c r="B64" s="7">
@@ -5611,7 +5611,7 @@
       </c>
     </row>
     <row r="65" spans="1:28">
-      <c r="A65" s="50"/>
+      <c r="A65" s="69"/>
       <c r="B65" s="3">
         <v>46175</v>
       </c>
@@ -5682,7 +5682,7 @@
       </c>
     </row>
     <row r="66" spans="1:28">
-      <c r="A66" s="50"/>
+      <c r="A66" s="69"/>
       <c r="B66" s="3">
         <v>46176</v>
       </c>
@@ -5753,7 +5753,7 @@
       </c>
     </row>
     <row r="67" spans="1:28">
-      <c r="A67" s="50"/>
+      <c r="A67" s="69"/>
       <c r="B67" s="3">
         <v>46177</v>
       </c>
@@ -5824,7 +5824,7 @@
       </c>
     </row>
     <row r="68" spans="1:28">
-      <c r="A68" s="50"/>
+      <c r="A68" s="69"/>
       <c r="B68" s="3">
         <v>46178</v>
       </c>
@@ -5895,7 +5895,7 @@
       </c>
     </row>
     <row r="69" spans="1:28">
-      <c r="A69" s="50"/>
+      <c r="A69" s="69"/>
       <c r="B69" s="3">
         <v>46179</v>
       </c>
@@ -5966,7 +5966,7 @@
       </c>
     </row>
     <row r="70" spans="1:28">
-      <c r="A70" s="50"/>
+      <c r="A70" s="69"/>
       <c r="B70" s="3">
         <v>46180</v>
       </c>
@@ -6037,7 +6037,7 @@
       </c>
     </row>
     <row r="71" spans="1:28">
-      <c r="A71" s="50"/>
+      <c r="A71" s="69"/>
       <c r="B71" s="3">
         <v>46181</v>
       </c>
@@ -6108,7 +6108,7 @@
       </c>
     </row>
     <row r="72" spans="1:28">
-      <c r="A72" s="50"/>
+      <c r="A72" s="69"/>
       <c r="B72" s="3">
         <v>46182</v>
       </c>
@@ -6179,7 +6179,7 @@
       </c>
     </row>
     <row r="73" spans="1:28">
-      <c r="A73" s="50"/>
+      <c r="A73" s="69"/>
       <c r="B73" s="3">
         <v>46183</v>
       </c>
@@ -6250,7 +6250,7 @@
       </c>
     </row>
     <row r="74" spans="1:28">
-      <c r="A74" s="50"/>
+      <c r="A74" s="69"/>
       <c r="B74" s="3">
         <v>46184</v>
       </c>
@@ -6321,7 +6321,7 @@
       </c>
     </row>
     <row r="75" spans="1:28">
-      <c r="A75" s="50"/>
+      <c r="A75" s="69"/>
       <c r="B75" s="3">
         <v>46185</v>
       </c>
@@ -6392,7 +6392,7 @@
       </c>
     </row>
     <row r="76" spans="1:28">
-      <c r="A76" s="50"/>
+      <c r="A76" s="69"/>
       <c r="B76" s="3">
         <v>46186</v>
       </c>
@@ -6463,7 +6463,7 @@
       </c>
     </row>
     <row r="77" spans="1:28">
-      <c r="A77" s="50"/>
+      <c r="A77" s="69"/>
       <c r="B77" s="3">
         <v>46187</v>
       </c>
@@ -6534,7 +6534,7 @@
       </c>
     </row>
     <row r="78" spans="1:28">
-      <c r="A78" s="50"/>
+      <c r="A78" s="69"/>
       <c r="B78" s="3">
         <v>46188</v>
       </c>
@@ -6605,7 +6605,7 @@
       </c>
     </row>
     <row r="79" spans="1:28">
-      <c r="A79" s="50"/>
+      <c r="A79" s="69"/>
       <c r="B79" s="3">
         <v>46189</v>
       </c>
@@ -6676,7 +6676,7 @@
       </c>
     </row>
     <row r="80" spans="1:28">
-      <c r="A80" s="50"/>
+      <c r="A80" s="69"/>
       <c r="B80" s="3">
         <v>46190</v>
       </c>
@@ -6747,7 +6747,7 @@
       </c>
     </row>
     <row r="81" spans="1:28">
-      <c r="A81" s="50"/>
+      <c r="A81" s="69"/>
       <c r="B81" s="3">
         <v>46191</v>
       </c>
@@ -6818,7 +6818,7 @@
       </c>
     </row>
     <row r="82" spans="1:28">
-      <c r="A82" s="50"/>
+      <c r="A82" s="69"/>
       <c r="B82" s="3">
         <v>46192</v>
       </c>
@@ -6889,7 +6889,7 @@
       </c>
     </row>
     <row r="83" spans="1:28">
-      <c r="A83" s="50"/>
+      <c r="A83" s="69"/>
       <c r="B83" s="3">
         <v>46193</v>
       </c>
@@ -6960,7 +6960,7 @@
       </c>
     </row>
     <row r="84" spans="1:28">
-      <c r="A84" s="50"/>
+      <c r="A84" s="69"/>
       <c r="B84" s="3">
         <v>46194</v>
       </c>
@@ -7031,7 +7031,7 @@
       </c>
     </row>
     <row r="85" spans="1:28">
-      <c r="A85" s="50"/>
+      <c r="A85" s="69"/>
       <c r="B85" s="3">
         <v>46195</v>
       </c>
@@ -7102,7 +7102,7 @@
       </c>
     </row>
     <row r="86" spans="1:28">
-      <c r="A86" s="50"/>
+      <c r="A86" s="69"/>
       <c r="B86" s="3">
         <v>46196</v>
       </c>
@@ -7173,7 +7173,7 @@
       </c>
     </row>
     <row r="87" spans="1:28">
-      <c r="A87" s="50"/>
+      <c r="A87" s="69"/>
       <c r="B87" s="3">
         <v>46197</v>
       </c>
@@ -7244,7 +7244,7 @@
       </c>
     </row>
     <row r="88" spans="1:28">
-      <c r="A88" s="50"/>
+      <c r="A88" s="69"/>
       <c r="B88" s="3">
         <v>46198</v>
       </c>
@@ -7315,7 +7315,7 @@
       </c>
     </row>
     <row r="89" spans="1:28">
-      <c r="A89" s="50"/>
+      <c r="A89" s="69"/>
       <c r="B89" s="3">
         <v>46199</v>
       </c>
@@ -7386,7 +7386,7 @@
       </c>
     </row>
     <row r="90" spans="1:28">
-      <c r="A90" s="50"/>
+      <c r="A90" s="69"/>
       <c r="B90" s="3">
         <v>46200</v>
       </c>
@@ -7457,7 +7457,7 @@
       </c>
     </row>
     <row r="91" spans="1:28">
-      <c r="A91" s="50"/>
+      <c r="A91" s="69"/>
       <c r="B91" s="3">
         <v>46201</v>
       </c>
@@ -7528,7 +7528,7 @@
       </c>
     </row>
     <row r="92" spans="1:28">
-      <c r="A92" s="50"/>
+      <c r="A92" s="69"/>
       <c r="B92" s="3">
         <v>46202</v>
       </c>
@@ -7599,7 +7599,7 @@
       </c>
     </row>
     <row r="93" spans="1:28" ht="15.75" thickBot="1">
-      <c r="A93" s="51"/>
+      <c r="A93" s="70"/>
       <c r="B93" s="3">
         <v>46203</v>
       </c>
@@ -7670,7 +7670,7 @@
       </c>
     </row>
     <row r="94" spans="1:28" ht="15.75" customHeight="1">
-      <c r="A94" s="52" t="s">
+      <c r="A94" s="71" t="s">
         <v>32</v>
       </c>
       <c r="B94" s="7">
@@ -7743,7 +7743,7 @@
       </c>
     </row>
     <row r="95" spans="1:28">
-      <c r="A95" s="53"/>
+      <c r="A95" s="72"/>
       <c r="B95" s="3">
         <v>46205</v>
       </c>
@@ -7814,7 +7814,7 @@
       </c>
     </row>
     <row r="96" spans="1:28">
-      <c r="A96" s="53"/>
+      <c r="A96" s="72"/>
       <c r="B96" s="3">
         <v>46206</v>
       </c>
@@ -7885,7 +7885,7 @@
       </c>
     </row>
     <row r="97" spans="1:28">
-      <c r="A97" s="53"/>
+      <c r="A97" s="72"/>
       <c r="B97" s="3">
         <v>46207</v>
       </c>
@@ -7956,7 +7956,7 @@
       </c>
     </row>
     <row r="98" spans="1:28">
-      <c r="A98" s="53"/>
+      <c r="A98" s="72"/>
       <c r="B98" s="3">
         <v>46208</v>
       </c>
@@ -8027,7 +8027,7 @@
       </c>
     </row>
     <row r="99" spans="1:28">
-      <c r="A99" s="53"/>
+      <c r="A99" s="72"/>
       <c r="B99" s="3">
         <v>46209</v>
       </c>
@@ -8098,7 +8098,7 @@
       </c>
     </row>
     <row r="100" spans="1:28">
-      <c r="A100" s="53"/>
+      <c r="A100" s="72"/>
       <c r="B100" s="3">
         <v>46210</v>
       </c>
@@ -8169,7 +8169,7 @@
       </c>
     </row>
     <row r="101" spans="1:28">
-      <c r="A101" s="53"/>
+      <c r="A101" s="72"/>
       <c r="B101" s="3">
         <v>46211</v>
       </c>
@@ -8240,7 +8240,7 @@
       </c>
     </row>
     <row r="102" spans="1:28">
-      <c r="A102" s="53"/>
+      <c r="A102" s="72"/>
       <c r="B102" s="3">
         <v>46212</v>
       </c>
@@ -8311,7 +8311,7 @@
       </c>
     </row>
     <row r="103" spans="1:28">
-      <c r="A103" s="53"/>
+      <c r="A103" s="72"/>
       <c r="B103" s="3">
         <v>46213</v>
       </c>
@@ -8382,7 +8382,7 @@
       </c>
     </row>
     <row r="104" spans="1:28">
-      <c r="A104" s="53"/>
+      <c r="A104" s="72"/>
       <c r="B104" s="3">
         <v>46214</v>
       </c>
@@ -8453,7 +8453,7 @@
       </c>
     </row>
     <row r="105" spans="1:28">
-      <c r="A105" s="53"/>
+      <c r="A105" s="72"/>
       <c r="B105" s="3">
         <v>46215</v>
       </c>
@@ -8524,7 +8524,7 @@
       </c>
     </row>
     <row r="106" spans="1:28">
-      <c r="A106" s="53"/>
+      <c r="A106" s="72"/>
       <c r="B106" s="3">
         <v>46216</v>
       </c>
@@ -8595,7 +8595,7 @@
       </c>
     </row>
     <row r="107" spans="1:28">
-      <c r="A107" s="53"/>
+      <c r="A107" s="72"/>
       <c r="B107" s="3">
         <v>46217</v>
       </c>
@@ -8666,7 +8666,7 @@
       </c>
     </row>
     <row r="108" spans="1:28">
-      <c r="A108" s="53"/>
+      <c r="A108" s="72"/>
       <c r="B108" s="3">
         <v>46218</v>
       </c>
@@ -8737,7 +8737,7 @@
       </c>
     </row>
     <row r="109" spans="1:28">
-      <c r="A109" s="53"/>
+      <c r="A109" s="72"/>
       <c r="B109" s="3">
         <v>46219</v>
       </c>
@@ -8808,7 +8808,7 @@
       </c>
     </row>
     <row r="110" spans="1:28">
-      <c r="A110" s="53"/>
+      <c r="A110" s="72"/>
       <c r="B110" s="3">
         <v>46220</v>
       </c>
@@ -8879,7 +8879,7 @@
       </c>
     </row>
     <row r="111" spans="1:28">
-      <c r="A111" s="53"/>
+      <c r="A111" s="72"/>
       <c r="B111" s="3">
         <v>46221</v>
       </c>
@@ -8950,7 +8950,7 @@
       </c>
     </row>
     <row r="112" spans="1:28">
-      <c r="A112" s="53"/>
+      <c r="A112" s="72"/>
       <c r="B112" s="3">
         <v>46222</v>
       </c>
@@ -9021,7 +9021,7 @@
       </c>
     </row>
     <row r="113" spans="1:28">
-      <c r="A113" s="53"/>
+      <c r="A113" s="72"/>
       <c r="B113" s="3">
         <v>46223</v>
       </c>
@@ -9092,7 +9092,7 @@
       </c>
     </row>
     <row r="114" spans="1:28">
-      <c r="A114" s="53"/>
+      <c r="A114" s="72"/>
       <c r="B114" s="3">
         <v>46224</v>
       </c>
@@ -9163,7 +9163,7 @@
       </c>
     </row>
     <row r="115" spans="1:28">
-      <c r="A115" s="53"/>
+      <c r="A115" s="72"/>
       <c r="B115" s="3">
         <v>46225</v>
       </c>
@@ -9234,7 +9234,7 @@
       </c>
     </row>
     <row r="116" spans="1:28">
-      <c r="A116" s="53"/>
+      <c r="A116" s="72"/>
       <c r="B116" s="3">
         <v>46226</v>
       </c>
@@ -9305,7 +9305,7 @@
       </c>
     </row>
     <row r="117" spans="1:28">
-      <c r="A117" s="53"/>
+      <c r="A117" s="72"/>
       <c r="B117" s="3">
         <v>46227</v>
       </c>
@@ -9376,7 +9376,7 @@
       </c>
     </row>
     <row r="118" spans="1:28">
-      <c r="A118" s="53"/>
+      <c r="A118" s="72"/>
       <c r="B118" s="3">
         <v>46228</v>
       </c>
@@ -9447,7 +9447,7 @@
       </c>
     </row>
     <row r="119" spans="1:28">
-      <c r="A119" s="53"/>
+      <c r="A119" s="72"/>
       <c r="B119" s="3">
         <v>46229</v>
       </c>
@@ -9518,7 +9518,7 @@
       </c>
     </row>
     <row r="120" spans="1:28">
-      <c r="A120" s="53"/>
+      <c r="A120" s="72"/>
       <c r="B120" s="3">
         <v>46230</v>
       </c>
@@ -9589,7 +9589,7 @@
       </c>
     </row>
     <row r="121" spans="1:28">
-      <c r="A121" s="53"/>
+      <c r="A121" s="72"/>
       <c r="B121" s="3">
         <v>46231</v>
       </c>
@@ -9660,7 +9660,7 @@
       </c>
     </row>
     <row r="122" spans="1:28">
-      <c r="A122" s="53"/>
+      <c r="A122" s="72"/>
       <c r="B122" s="3">
         <v>46232</v>
       </c>
@@ -9731,7 +9731,7 @@
       </c>
     </row>
     <row r="123" spans="1:28">
-      <c r="A123" s="53"/>
+      <c r="A123" s="72"/>
       <c r="B123" s="3">
         <v>46233</v>
       </c>
@@ -9802,7 +9802,7 @@
       </c>
     </row>
     <row r="124" spans="1:28" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A124" s="53"/>
+      <c r="A124" s="72"/>
       <c r="B124" s="3">
         <v>46234</v>
       </c>
@@ -9873,7 +9873,7 @@
       </c>
     </row>
     <row r="125" spans="1:28">
-      <c r="A125" s="54" t="s">
+      <c r="A125" s="73" t="s">
         <v>33</v>
       </c>
       <c r="B125" s="7">
@@ -9946,7 +9946,7 @@
       </c>
     </row>
     <row r="126" spans="1:28">
-      <c r="A126" s="54"/>
+      <c r="A126" s="73"/>
       <c r="B126" s="3">
         <v>46236</v>
       </c>
@@ -10017,7 +10017,7 @@
       </c>
     </row>
     <row r="127" spans="1:28">
-      <c r="A127" s="54"/>
+      <c r="A127" s="73"/>
       <c r="B127" s="3">
         <v>46237</v>
       </c>
@@ -10088,7 +10088,7 @@
       </c>
     </row>
     <row r="128" spans="1:28">
-      <c r="A128" s="54"/>
+      <c r="A128" s="73"/>
       <c r="B128" s="3">
         <v>46238</v>
       </c>
@@ -10161,7 +10161,7 @@
       </c>
     </row>
     <row r="129" spans="1:28">
-      <c r="A129" s="54"/>
+      <c r="A129" s="73"/>
       <c r="B129" s="3">
         <v>46239</v>
       </c>
@@ -10234,7 +10234,7 @@
       </c>
     </row>
     <row r="130" spans="1:28">
-      <c r="A130" s="54"/>
+      <c r="A130" s="73"/>
       <c r="B130" s="3">
         <v>46240</v>
       </c>
@@ -10307,7 +10307,7 @@
       </c>
     </row>
     <row r="131" spans="1:28">
-      <c r="A131" s="54"/>
+      <c r="A131" s="73"/>
       <c r="B131" s="3">
         <v>46241</v>
       </c>
@@ -10380,7 +10380,7 @@
       </c>
     </row>
     <row r="132" spans="1:28">
-      <c r="A132" s="54"/>
+      <c r="A132" s="73"/>
       <c r="B132" s="3">
         <v>46242</v>
       </c>
@@ -10453,7 +10453,7 @@
       </c>
     </row>
     <row r="133" spans="1:28">
-      <c r="A133" s="54"/>
+      <c r="A133" s="73"/>
       <c r="B133" s="3">
         <v>46243</v>
       </c>
@@ -10526,7 +10526,7 @@
       </c>
     </row>
     <row r="134" spans="1:28">
-      <c r="A134" s="54"/>
+      <c r="A134" s="73"/>
       <c r="B134" s="3">
         <v>46244</v>
       </c>
@@ -10599,7 +10599,7 @@
       </c>
     </row>
     <row r="135" spans="1:28">
-      <c r="A135" s="54"/>
+      <c r="A135" s="73"/>
       <c r="B135" s="3">
         <v>46245</v>
       </c>
@@ -10672,7 +10672,7 @@
       </c>
     </row>
     <row r="136" spans="1:28">
-      <c r="A136" s="54"/>
+      <c r="A136" s="73"/>
       <c r="B136" s="3">
         <v>46246</v>
       </c>
@@ -10745,7 +10745,7 @@
       </c>
     </row>
     <row r="137" spans="1:28">
-      <c r="A137" s="54"/>
+      <c r="A137" s="73"/>
       <c r="B137" s="3">
         <v>46247</v>
       </c>
@@ -10818,7 +10818,7 @@
       </c>
     </row>
     <row r="138" spans="1:28">
-      <c r="A138" s="54"/>
+      <c r="A138" s="73"/>
       <c r="B138" s="3">
         <v>46248</v>
       </c>
@@ -10891,7 +10891,7 @@
       </c>
     </row>
     <row r="139" spans="1:28">
-      <c r="A139" s="54"/>
+      <c r="A139" s="73"/>
       <c r="B139" s="3">
         <v>46249</v>
       </c>
@@ -10964,7 +10964,7 @@
       </c>
     </row>
     <row r="140" spans="1:28">
-      <c r="A140" s="54"/>
+      <c r="A140" s="73"/>
       <c r="B140" s="3">
         <v>46250</v>
       </c>
@@ -11037,7 +11037,7 @@
       </c>
     </row>
     <row r="141" spans="1:28">
-      <c r="A141" s="54"/>
+      <c r="A141" s="73"/>
       <c r="B141" s="3">
         <v>46251</v>
       </c>
@@ -11110,7 +11110,7 @@
       </c>
     </row>
     <row r="142" spans="1:28">
-      <c r="A142" s="54"/>
+      <c r="A142" s="73"/>
       <c r="B142" s="3">
         <v>46252</v>
       </c>
@@ -11183,7 +11183,7 @@
       </c>
     </row>
     <row r="143" spans="1:28">
-      <c r="A143" s="54"/>
+      <c r="A143" s="73"/>
       <c r="B143" s="3">
         <v>46253</v>
       </c>
@@ -11256,7 +11256,7 @@
       </c>
     </row>
     <row r="144" spans="1:28">
-      <c r="A144" s="54"/>
+      <c r="A144" s="73"/>
       <c r="B144" s="3">
         <v>46254</v>
       </c>
@@ -11329,7 +11329,7 @@
       </c>
     </row>
     <row r="145" spans="1:28">
-      <c r="A145" s="54"/>
+      <c r="A145" s="73"/>
       <c r="B145" s="3">
         <v>46255</v>
       </c>
@@ -11402,7 +11402,7 @@
       </c>
     </row>
     <row r="146" spans="1:28">
-      <c r="A146" s="54"/>
+      <c r="A146" s="73"/>
       <c r="B146" s="3">
         <v>46256</v>
       </c>
@@ -11475,7 +11475,7 @@
       </c>
     </row>
     <row r="147" spans="1:28">
-      <c r="A147" s="54"/>
+      <c r="A147" s="73"/>
       <c r="B147" s="3">
         <v>46257</v>
       </c>
@@ -11548,7 +11548,7 @@
       </c>
     </row>
     <row r="148" spans="1:28">
-      <c r="A148" s="54"/>
+      <c r="A148" s="73"/>
       <c r="B148" s="3">
         <v>46258</v>
       </c>
@@ -11621,7 +11621,7 @@
       </c>
     </row>
     <row r="149" spans="1:28">
-      <c r="A149" s="54"/>
+      <c r="A149" s="73"/>
       <c r="B149" s="3">
         <v>46259</v>
       </c>
@@ -11694,7 +11694,7 @@
       </c>
     </row>
     <row r="150" spans="1:28">
-      <c r="A150" s="54"/>
+      <c r="A150" s="73"/>
       <c r="B150" s="3">
         <v>46260</v>
       </c>
@@ -11767,7 +11767,7 @@
       </c>
     </row>
     <row r="151" spans="1:28">
-      <c r="A151" s="54"/>
+      <c r="A151" s="73"/>
       <c r="B151" s="3">
         <v>46261</v>
       </c>
@@ -11842,7 +11842,7 @@
       </c>
     </row>
     <row r="152" spans="1:28">
-      <c r="A152" s="54"/>
+      <c r="A152" s="73"/>
       <c r="B152" s="3">
         <v>46262</v>
       </c>
@@ -11917,7 +11917,7 @@
       </c>
     </row>
     <row r="153" spans="1:28">
-      <c r="A153" s="54"/>
+      <c r="A153" s="73"/>
       <c r="B153" s="3">
         <v>46263</v>
       </c>
@@ -11992,7 +11992,7 @@
       </c>
     </row>
     <row r="154" spans="1:28">
-      <c r="A154" s="54"/>
+      <c r="A154" s="73"/>
       <c r="B154" s="3">
         <v>46264</v>
       </c>
@@ -12067,7 +12067,7 @@
       </c>
     </row>
     <row r="155" spans="1:28" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A155" s="54"/>
+      <c r="A155" s="73"/>
       <c r="B155" s="3">
         <v>46265</v>
       </c>
@@ -12142,7 +12142,7 @@
       </c>
     </row>
     <row r="156" spans="1:28">
-      <c r="A156" s="54" t="s">
+      <c r="A156" s="73" t="s">
         <v>34</v>
       </c>
       <c r="B156" s="7">
@@ -12219,7 +12219,7 @@
       </c>
     </row>
     <row r="157" spans="1:28">
-      <c r="A157" s="54"/>
+      <c r="A157" s="73"/>
       <c r="B157" s="3">
         <v>46267</v>
       </c>
@@ -12294,7 +12294,7 @@
       </c>
     </row>
     <row r="158" spans="1:28">
-      <c r="A158" s="54"/>
+      <c r="A158" s="73"/>
       <c r="B158" s="3">
         <v>46268</v>
       </c>
@@ -12369,7 +12369,7 @@
       </c>
     </row>
     <row r="159" spans="1:28">
-      <c r="A159" s="54"/>
+      <c r="A159" s="73"/>
       <c r="B159" s="3">
         <v>46269</v>
       </c>
@@ -12444,7 +12444,7 @@
       </c>
     </row>
     <row r="160" spans="1:28">
-      <c r="A160" s="54"/>
+      <c r="A160" s="73"/>
       <c r="B160" s="3">
         <v>46270</v>
       </c>
@@ -12519,7 +12519,7 @@
       </c>
     </row>
     <row r="161" spans="1:28">
-      <c r="A161" s="54"/>
+      <c r="A161" s="73"/>
       <c r="B161" s="3">
         <v>46271</v>
       </c>
@@ -12594,7 +12594,7 @@
       </c>
     </row>
     <row r="162" spans="1:28">
-      <c r="A162" s="54"/>
+      <c r="A162" s="73"/>
       <c r="B162" s="3">
         <v>46272</v>
       </c>
@@ -12669,7 +12669,7 @@
       </c>
     </row>
     <row r="163" spans="1:28">
-      <c r="A163" s="54"/>
+      <c r="A163" s="73"/>
       <c r="B163" s="3">
         <v>46273</v>
       </c>
@@ -12744,7 +12744,7 @@
       </c>
     </row>
     <row r="164" spans="1:28">
-      <c r="A164" s="54"/>
+      <c r="A164" s="73"/>
       <c r="B164" s="3">
         <v>46274</v>
       </c>
@@ -12819,7 +12819,7 @@
       </c>
     </row>
     <row r="165" spans="1:28">
-      <c r="A165" s="54"/>
+      <c r="A165" s="73"/>
       <c r="B165" s="3">
         <v>46275</v>
       </c>
@@ -12896,7 +12896,7 @@
       </c>
     </row>
     <row r="166" spans="1:28">
-      <c r="A166" s="54"/>
+      <c r="A166" s="73"/>
       <c r="B166" s="3">
         <v>46276</v>
       </c>
@@ -12973,7 +12973,7 @@
       </c>
     </row>
     <row r="167" spans="1:28">
-      <c r="A167" s="54"/>
+      <c r="A167" s="73"/>
       <c r="B167" s="3">
         <v>46277</v>
       </c>
@@ -13050,7 +13050,7 @@
       </c>
     </row>
     <row r="168" spans="1:28">
-      <c r="A168" s="54"/>
+      <c r="A168" s="73"/>
       <c r="B168" s="3">
         <v>46278</v>
       </c>
@@ -13129,7 +13129,7 @@
       </c>
     </row>
     <row r="169" spans="1:28">
-      <c r="A169" s="54"/>
+      <c r="A169" s="73"/>
       <c r="B169" s="3">
         <v>46279</v>
       </c>
@@ -13208,7 +13208,7 @@
       </c>
     </row>
     <row r="170" spans="1:28">
-      <c r="A170" s="54"/>
+      <c r="A170" s="73"/>
       <c r="B170" s="3">
         <v>46280</v>
       </c>
@@ -13287,7 +13287,7 @@
       </c>
     </row>
     <row r="171" spans="1:28">
-      <c r="A171" s="54"/>
+      <c r="A171" s="73"/>
       <c r="B171" s="3">
         <v>46281</v>
       </c>
@@ -13366,7 +13366,7 @@
       </c>
     </row>
     <row r="172" spans="1:28">
-      <c r="A172" s="54"/>
+      <c r="A172" s="73"/>
       <c r="B172" s="3">
         <v>46282</v>
       </c>
@@ -13445,7 +13445,7 @@
       </c>
     </row>
     <row r="173" spans="1:28">
-      <c r="A173" s="54"/>
+      <c r="A173" s="73"/>
       <c r="B173" s="3">
         <v>46283</v>
       </c>
@@ -13524,7 +13524,7 @@
       </c>
     </row>
     <row r="174" spans="1:28">
-      <c r="A174" s="54"/>
+      <c r="A174" s="73"/>
       <c r="B174" s="3">
         <v>46284</v>
       </c>
@@ -13603,7 +13603,7 @@
       </c>
     </row>
     <row r="175" spans="1:28">
-      <c r="A175" s="54"/>
+      <c r="A175" s="73"/>
       <c r="B175" s="3">
         <v>46285</v>
       </c>
@@ -13682,7 +13682,7 @@
       </c>
     </row>
     <row r="176" spans="1:28">
-      <c r="A176" s="54"/>
+      <c r="A176" s="73"/>
       <c r="B176" s="3">
         <v>46286</v>
       </c>
@@ -13761,7 +13761,7 @@
       </c>
     </row>
     <row r="177" spans="1:28">
-      <c r="A177" s="54"/>
+      <c r="A177" s="73"/>
       <c r="B177" s="3">
         <v>46287</v>
       </c>
@@ -13840,7 +13840,7 @@
       </c>
     </row>
     <row r="178" spans="1:28">
-      <c r="A178" s="54"/>
+      <c r="A178" s="73"/>
       <c r="B178" s="3">
         <v>46288</v>
       </c>
@@ -13919,7 +13919,7 @@
       </c>
     </row>
     <row r="179" spans="1:28">
-      <c r="A179" s="54"/>
+      <c r="A179" s="73"/>
       <c r="B179" s="3">
         <v>46289</v>
       </c>
@@ -13998,7 +13998,7 @@
       </c>
     </row>
     <row r="180" spans="1:28">
-      <c r="A180" s="54"/>
+      <c r="A180" s="73"/>
       <c r="B180" s="3">
         <v>46290</v>
       </c>
@@ -14077,7 +14077,7 @@
       </c>
     </row>
     <row r="181" spans="1:28">
-      <c r="A181" s="54"/>
+      <c r="A181" s="73"/>
       <c r="B181" s="3">
         <v>46291</v>
       </c>
@@ -14156,7 +14156,7 @@
       </c>
     </row>
     <row r="182" spans="1:28">
-      <c r="A182" s="54"/>
+      <c r="A182" s="73"/>
       <c r="B182" s="3">
         <v>46292</v>
       </c>
@@ -14235,7 +14235,7 @@
       </c>
     </row>
     <row r="183" spans="1:28">
-      <c r="A183" s="54"/>
+      <c r="A183" s="73"/>
       <c r="B183" s="3">
         <v>46293</v>
       </c>
@@ -14314,7 +14314,7 @@
       </c>
     </row>
     <row r="184" spans="1:28">
-      <c r="A184" s="54"/>
+      <c r="A184" s="73"/>
       <c r="B184" s="3">
         <v>46294</v>
       </c>
@@ -14393,7 +14393,7 @@
       </c>
     </row>
     <row r="185" spans="1:28">
-      <c r="A185" s="54"/>
+      <c r="A185" s="73"/>
       <c r="B185" s="18">
         <v>46295</v>
       </c>
@@ -14472,7 +14472,7 @@
       </c>
     </row>
     <row r="186" spans="1:28" ht="15" customHeight="1">
-      <c r="A186" s="68" t="s">
+      <c r="A186" s="56" t="s">
         <v>40</v>
       </c>
       <c r="B186" s="30">
@@ -14553,7 +14553,7 @@
       </c>
     </row>
     <row r="187" spans="1:28">
-      <c r="A187" s="69"/>
+      <c r="A187" s="57"/>
       <c r="B187" s="3">
         <v>46297</v>
       </c>
@@ -14632,7 +14632,7 @@
       </c>
     </row>
     <row r="188" spans="1:28">
-      <c r="A188" s="69"/>
+      <c r="A188" s="57"/>
       <c r="B188" s="3">
         <v>46298</v>
       </c>
@@ -14711,7 +14711,7 @@
       </c>
     </row>
     <row r="189" spans="1:28">
-      <c r="A189" s="69"/>
+      <c r="A189" s="57"/>
       <c r="B189" s="3">
         <v>46299</v>
       </c>
@@ -14790,7 +14790,7 @@
       </c>
     </row>
     <row r="190" spans="1:28">
-      <c r="A190" s="69"/>
+      <c r="A190" s="57"/>
       <c r="B190" s="3">
         <v>46300</v>
       </c>
@@ -14869,7 +14869,7 @@
       </c>
     </row>
     <row r="191" spans="1:28">
-      <c r="A191" s="69"/>
+      <c r="A191" s="57"/>
       <c r="B191" s="3">
         <v>46301</v>
       </c>
@@ -14948,7 +14948,7 @@
       </c>
     </row>
     <row r="192" spans="1:28">
-      <c r="A192" s="69"/>
+      <c r="A192" s="57"/>
       <c r="B192" s="3">
         <v>46302</v>
       </c>
@@ -15027,7 +15027,7 @@
       </c>
     </row>
     <row r="193" spans="1:28">
-      <c r="A193" s="69"/>
+      <c r="A193" s="57"/>
       <c r="B193" s="3">
         <v>46303</v>
       </c>
@@ -15106,7 +15106,7 @@
       </c>
     </row>
     <row r="194" spans="1:28">
-      <c r="A194" s="69"/>
+      <c r="A194" s="57"/>
       <c r="B194" s="3">
         <v>46304</v>
       </c>
@@ -15185,7 +15185,7 @@
       </c>
     </row>
     <row r="195" spans="1:28">
-      <c r="A195" s="69"/>
+      <c r="A195" s="57"/>
       <c r="B195" s="3">
         <v>46305</v>
       </c>
@@ -15264,7 +15264,7 @@
       </c>
     </row>
     <row r="196" spans="1:28">
-      <c r="A196" s="69"/>
+      <c r="A196" s="57"/>
       <c r="B196" s="3">
         <v>46306</v>
       </c>
@@ -15343,7 +15343,7 @@
       </c>
     </row>
     <row r="197" spans="1:28">
-      <c r="A197" s="69"/>
+      <c r="A197" s="57"/>
       <c r="B197" s="3">
         <v>46307</v>
       </c>
@@ -15418,7 +15418,7 @@
       </c>
     </row>
     <row r="198" spans="1:28">
-      <c r="A198" s="69"/>
+      <c r="A198" s="57"/>
       <c r="B198" s="3">
         <v>46308</v>
       </c>
@@ -15493,7 +15493,7 @@
       </c>
     </row>
     <row r="199" spans="1:28">
-      <c r="A199" s="69"/>
+      <c r="A199" s="57"/>
       <c r="B199" s="3">
         <v>46309</v>
       </c>
@@ -15568,7 +15568,7 @@
       </c>
     </row>
     <row r="200" spans="1:28">
-      <c r="A200" s="69"/>
+      <c r="A200" s="57"/>
       <c r="B200" s="3">
         <v>46310</v>
       </c>
@@ -15643,7 +15643,7 @@
       </c>
     </row>
     <row r="201" spans="1:28">
-      <c r="A201" s="69"/>
+      <c r="A201" s="57"/>
       <c r="B201" s="3">
         <v>46311</v>
       </c>
@@ -15724,7 +15724,7 @@
       </c>
     </row>
     <row r="202" spans="1:28">
-      <c r="A202" s="69"/>
+      <c r="A202" s="57"/>
       <c r="B202" s="3">
         <v>46312</v>
       </c>
@@ -15747,7 +15747,7 @@
         <v>24</v>
       </c>
       <c r="K202" s="4">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="L202" s="5"/>
       <c r="M202" s="5"/>
@@ -15783,19 +15783,31 @@
       </c>
     </row>
     <row r="203" spans="1:28">
-      <c r="A203" s="69"/>
+      <c r="A203" s="57"/>
       <c r="B203" s="3">
         <v>46313</v>
       </c>
       <c r="C203" s="4"/>
       <c r="D203" s="4"/>
       <c r="E203" s="4"/>
-      <c r="F203" s="5"/>
-      <c r="G203" s="5"/>
-      <c r="H203" s="5"/>
-      <c r="I203" s="4"/>
-      <c r="J203" s="4"/>
-      <c r="K203" s="4"/>
+      <c r="F203" s="5">
+        <v>24</v>
+      </c>
+      <c r="G203" s="5">
+        <v>24</v>
+      </c>
+      <c r="H203" s="5">
+        <v>24</v>
+      </c>
+      <c r="I203" s="4">
+        <v>24</v>
+      </c>
+      <c r="J203" s="4">
+        <v>24</v>
+      </c>
+      <c r="K203" s="4">
+        <v>14</v>
+      </c>
       <c r="L203" s="5"/>
       <c r="M203" s="5"/>
       <c r="N203" s="5"/>
@@ -15830,7 +15842,7 @@
       </c>
     </row>
     <row r="204" spans="1:28">
-      <c r="A204" s="69"/>
+      <c r="A204" s="57"/>
       <c r="B204" s="3">
         <v>46314</v>
       </c>
@@ -15862,7 +15874,7 @@
       <c r="AB204" s="35"/>
     </row>
     <row r="205" spans="1:28">
-      <c r="A205" s="69"/>
+      <c r="A205" s="57"/>
       <c r="B205" s="3">
         <v>46315</v>
       </c>
@@ -15894,7 +15906,7 @@
       <c r="AB205" s="35"/>
     </row>
     <row r="206" spans="1:28">
-      <c r="A206" s="69"/>
+      <c r="A206" s="57"/>
       <c r="B206" s="3">
         <v>46316</v>
       </c>
@@ -15926,7 +15938,7 @@
       <c r="AB206" s="35"/>
     </row>
     <row r="207" spans="1:28">
-      <c r="A207" s="69"/>
+      <c r="A207" s="57"/>
       <c r="B207" s="3">
         <v>46317</v>
       </c>
@@ -15958,7 +15970,7 @@
       <c r="AB207" s="35"/>
     </row>
     <row r="208" spans="1:28">
-      <c r="A208" s="69"/>
+      <c r="A208" s="57"/>
       <c r="B208" s="3">
         <v>46318</v>
       </c>
@@ -15990,7 +16002,7 @@
       <c r="AB208" s="35"/>
     </row>
     <row r="209" spans="1:28">
-      <c r="A209" s="69"/>
+      <c r="A209" s="57"/>
       <c r="B209" s="3">
         <v>46319</v>
       </c>
@@ -16022,7 +16034,7 @@
       <c r="AB209" s="35"/>
     </row>
     <row r="210" spans="1:28">
-      <c r="A210" s="69"/>
+      <c r="A210" s="57"/>
       <c r="B210" s="3">
         <v>46320</v>
       </c>
@@ -16054,7 +16066,7 @@
       <c r="AB210" s="35"/>
     </row>
     <row r="211" spans="1:28">
-      <c r="A211" s="69"/>
+      <c r="A211" s="57"/>
       <c r="B211" s="3">
         <v>46321</v>
       </c>
@@ -16086,7 +16098,7 @@
       <c r="AB211" s="35"/>
     </row>
     <row r="212" spans="1:28">
-      <c r="A212" s="69"/>
+      <c r="A212" s="57"/>
       <c r="B212" s="3">
         <v>46322</v>
       </c>
@@ -16118,7 +16130,7 @@
       <c r="AB212" s="35"/>
     </row>
     <row r="213" spans="1:28">
-      <c r="A213" s="69"/>
+      <c r="A213" s="57"/>
       <c r="B213" s="18">
         <v>46323</v>
       </c>
@@ -16150,7 +16162,7 @@
       <c r="AB213" s="36"/>
     </row>
     <row r="214" spans="1:28">
-      <c r="A214" s="69"/>
+      <c r="A214" s="57"/>
       <c r="B214" s="24">
         <v>46324</v>
       </c>
@@ -16182,7 +16194,7 @@
       <c r="AB214" s="37"/>
     </row>
     <row r="215" spans="1:28">
-      <c r="A215" s="69"/>
+      <c r="A215" s="57"/>
       <c r="B215" s="24">
         <v>46325</v>
       </c>
@@ -16214,7 +16226,7 @@
       <c r="AB215" s="37"/>
     </row>
     <row r="216" spans="1:28">
-      <c r="A216" s="70"/>
+      <c r="A216" s="58"/>
       <c r="B216" s="38">
         <v>46326</v>
       </c>
@@ -16246,7 +16258,7 @@
       <c r="AB216" s="42"/>
     </row>
     <row r="217" spans="1:28">
-      <c r="A217" s="68" t="s">
+      <c r="A217" s="56" t="s">
         <v>35</v>
       </c>
       <c r="B217" s="30">
@@ -16280,7 +16292,7 @@
       <c r="AB217" s="34"/>
     </row>
     <row r="218" spans="1:28">
-      <c r="A218" s="69"/>
+      <c r="A218" s="57"/>
       <c r="B218" s="3">
         <v>46328</v>
       </c>
@@ -16312,7 +16324,7 @@
       <c r="AB218" s="35"/>
     </row>
     <row r="219" spans="1:28">
-      <c r="A219" s="69"/>
+      <c r="A219" s="57"/>
       <c r="B219" s="3">
         <v>46329</v>
       </c>
@@ -16344,7 +16356,7 @@
       <c r="AB219" s="35"/>
     </row>
     <row r="220" spans="1:28">
-      <c r="A220" s="69"/>
+      <c r="A220" s="57"/>
       <c r="B220" s="3">
         <v>46330</v>
       </c>
@@ -16376,7 +16388,7 @@
       <c r="AB220" s="35"/>
     </row>
     <row r="221" spans="1:28">
-      <c r="A221" s="69"/>
+      <c r="A221" s="57"/>
       <c r="B221" s="3">
         <v>46331</v>
       </c>
@@ -16408,7 +16420,7 @@
       <c r="AB221" s="35"/>
     </row>
     <row r="222" spans="1:28">
-      <c r="A222" s="69"/>
+      <c r="A222" s="57"/>
       <c r="B222" s="3">
         <v>46332</v>
       </c>
@@ -16440,7 +16452,7 @@
       <c r="AB222" s="35"/>
     </row>
     <row r="223" spans="1:28">
-      <c r="A223" s="69"/>
+      <c r="A223" s="57"/>
       <c r="B223" s="3">
         <v>46333</v>
       </c>
@@ -16472,7 +16484,7 @@
       <c r="AB223" s="35"/>
     </row>
     <row r="224" spans="1:28">
-      <c r="A224" s="69"/>
+      <c r="A224" s="57"/>
       <c r="B224" s="3">
         <v>46334</v>
       </c>
@@ -16504,7 +16516,7 @@
       <c r="AB224" s="35"/>
     </row>
     <row r="225" spans="1:28">
-      <c r="A225" s="69"/>
+      <c r="A225" s="57"/>
       <c r="B225" s="3">
         <v>46335</v>
       </c>
@@ -16536,7 +16548,7 @@
       <c r="AB225" s="35"/>
     </row>
     <row r="226" spans="1:28">
-      <c r="A226" s="69"/>
+      <c r="A226" s="57"/>
       <c r="B226" s="3">
         <v>46336</v>
       </c>
@@ -16568,7 +16580,7 @@
       <c r="AB226" s="35"/>
     </row>
     <row r="227" spans="1:28">
-      <c r="A227" s="69"/>
+      <c r="A227" s="57"/>
       <c r="B227" s="3">
         <v>46337</v>
       </c>
@@ -16600,7 +16612,7 @@
       <c r="AB227" s="35"/>
     </row>
     <row r="228" spans="1:28">
-      <c r="A228" s="69"/>
+      <c r="A228" s="57"/>
       <c r="B228" s="3">
         <v>46338</v>
       </c>
@@ -16632,7 +16644,7 @@
       <c r="AB228" s="35"/>
     </row>
     <row r="229" spans="1:28">
-      <c r="A229" s="69"/>
+      <c r="A229" s="57"/>
       <c r="B229" s="3">
         <v>46339</v>
       </c>
@@ -16664,7 +16676,7 @@
       <c r="AB229" s="35"/>
     </row>
     <row r="230" spans="1:28">
-      <c r="A230" s="69"/>
+      <c r="A230" s="57"/>
       <c r="B230" s="3">
         <v>46340</v>
       </c>
@@ -16696,7 +16708,7 @@
       <c r="AB230" s="35"/>
     </row>
     <row r="231" spans="1:28">
-      <c r="A231" s="69"/>
+      <c r="A231" s="57"/>
       <c r="B231" s="3">
         <v>46341</v>
       </c>
@@ -16728,7 +16740,7 @@
       <c r="AB231" s="35"/>
     </row>
     <row r="232" spans="1:28">
-      <c r="A232" s="69"/>
+      <c r="A232" s="57"/>
       <c r="B232" s="3">
         <v>46342</v>
       </c>
@@ -16760,7 +16772,7 @@
       <c r="AB232" s="35"/>
     </row>
     <row r="233" spans="1:28">
-      <c r="A233" s="69"/>
+      <c r="A233" s="57"/>
       <c r="B233" s="3">
         <v>46343</v>
       </c>
@@ -16792,7 +16804,7 @@
       <c r="AB233" s="35"/>
     </row>
     <row r="234" spans="1:28">
-      <c r="A234" s="69"/>
+      <c r="A234" s="57"/>
       <c r="B234" s="3">
         <v>46344</v>
       </c>
@@ -16824,7 +16836,7 @@
       <c r="AB234" s="35"/>
     </row>
     <row r="235" spans="1:28">
-      <c r="A235" s="69"/>
+      <c r="A235" s="57"/>
       <c r="B235" s="3">
         <v>46345</v>
       </c>
@@ -16856,7 +16868,7 @@
       <c r="AB235" s="35"/>
     </row>
     <row r="236" spans="1:28">
-      <c r="A236" s="69"/>
+      <c r="A236" s="57"/>
       <c r="B236" s="3">
         <v>46346</v>
       </c>
@@ -16888,7 +16900,7 @@
       <c r="AB236" s="35"/>
     </row>
     <row r="237" spans="1:28">
-      <c r="A237" s="69"/>
+      <c r="A237" s="57"/>
       <c r="B237" s="3">
         <v>46347</v>
       </c>
@@ -16920,7 +16932,7 @@
       <c r="AB237" s="35"/>
     </row>
     <row r="238" spans="1:28">
-      <c r="A238" s="69"/>
+      <c r="A238" s="57"/>
       <c r="B238" s="3">
         <v>46348</v>
       </c>
@@ -16952,7 +16964,7 @@
       <c r="AB238" s="35"/>
     </row>
     <row r="239" spans="1:28">
-      <c r="A239" s="69"/>
+      <c r="A239" s="57"/>
       <c r="B239" s="3">
         <v>46349</v>
       </c>
@@ -16984,7 +16996,7 @@
       <c r="AB239" s="35"/>
     </row>
     <row r="240" spans="1:28">
-      <c r="A240" s="69"/>
+      <c r="A240" s="57"/>
       <c r="B240" s="3">
         <v>46350</v>
       </c>
@@ -17016,7 +17028,7 @@
       <c r="AB240" s="35"/>
     </row>
     <row r="241" spans="1:28">
-      <c r="A241" s="69"/>
+      <c r="A241" s="57"/>
       <c r="B241" s="3">
         <v>46351</v>
       </c>
@@ -17048,7 +17060,7 @@
       <c r="AB241" s="35"/>
     </row>
     <row r="242" spans="1:28">
-      <c r="A242" s="69"/>
+      <c r="A242" s="57"/>
       <c r="B242" s="3">
         <v>46352</v>
       </c>
@@ -17080,7 +17092,7 @@
       <c r="AB242" s="35"/>
     </row>
     <row r="243" spans="1:28">
-      <c r="A243" s="69"/>
+      <c r="A243" s="57"/>
       <c r="B243" s="3">
         <v>46353</v>
       </c>
@@ -17112,7 +17124,7 @@
       <c r="AB243" s="35"/>
     </row>
     <row r="244" spans="1:28">
-      <c r="A244" s="69"/>
+      <c r="A244" s="57"/>
       <c r="B244" s="3">
         <v>46354</v>
       </c>
@@ -17144,7 +17156,7 @@
       <c r="AB244" s="35"/>
     </row>
     <row r="245" spans="1:28">
-      <c r="A245" s="69"/>
+      <c r="A245" s="57"/>
       <c r="B245" s="3">
         <v>46355</v>
       </c>
@@ -17176,7 +17188,7 @@
       <c r="AB245" s="35"/>
     </row>
     <row r="246" spans="1:28">
-      <c r="A246" s="70"/>
+      <c r="A246" s="58"/>
       <c r="B246" s="43">
         <v>46356</v>
       </c>
@@ -17208,7 +17220,7 @@
       <c r="AB246" s="47"/>
     </row>
     <row r="247" spans="1:28" ht="15" customHeight="1">
-      <c r="A247" s="67" t="s">
+      <c r="A247" s="55" t="s">
         <v>36</v>
       </c>
       <c r="B247" s="21">
@@ -17242,7 +17254,7 @@
       <c r="AB247" s="16"/>
     </row>
     <row r="248" spans="1:28" ht="15" customHeight="1">
-      <c r="A248" s="67"/>
+      <c r="A248" s="55"/>
       <c r="B248" s="3">
         <v>46358</v>
       </c>
@@ -17274,7 +17286,7 @@
       <c r="AB248" s="4"/>
     </row>
     <row r="249" spans="1:28" ht="15" customHeight="1">
-      <c r="A249" s="67"/>
+      <c r="A249" s="55"/>
       <c r="B249" s="3">
         <v>46359</v>
       </c>
@@ -17306,7 +17318,7 @@
       <c r="AB249" s="4"/>
     </row>
     <row r="250" spans="1:28" ht="15" customHeight="1">
-      <c r="A250" s="67"/>
+      <c r="A250" s="55"/>
       <c r="B250" s="3">
         <v>46360</v>
       </c>
@@ -17338,7 +17350,7 @@
       <c r="AB250" s="4"/>
     </row>
     <row r="251" spans="1:28" ht="15" customHeight="1">
-      <c r="A251" s="67"/>
+      <c r="A251" s="55"/>
       <c r="B251" s="3">
         <v>46361</v>
       </c>
@@ -17370,7 +17382,7 @@
       <c r="AB251" s="4"/>
     </row>
     <row r="252" spans="1:28" ht="15" customHeight="1">
-      <c r="A252" s="67"/>
+      <c r="A252" s="55"/>
       <c r="B252" s="3">
         <v>46362</v>
       </c>
@@ -17402,7 +17414,7 @@
       <c r="AB252" s="4"/>
     </row>
     <row r="253" spans="1:28" ht="15" customHeight="1">
-      <c r="A253" s="67"/>
+      <c r="A253" s="55"/>
       <c r="B253" s="3">
         <v>46363</v>
       </c>
@@ -17434,7 +17446,7 @@
       <c r="AB253" s="4"/>
     </row>
     <row r="254" spans="1:28" ht="15" customHeight="1">
-      <c r="A254" s="67"/>
+      <c r="A254" s="55"/>
       <c r="B254" s="3">
         <v>46364</v>
       </c>
@@ -17466,7 +17478,7 @@
       <c r="AB254" s="4"/>
     </row>
     <row r="255" spans="1:28" ht="15" customHeight="1">
-      <c r="A255" s="67"/>
+      <c r="A255" s="55"/>
       <c r="B255" s="3">
         <v>46365</v>
       </c>
@@ -17498,7 +17510,7 @@
       <c r="AB255" s="4"/>
     </row>
     <row r="256" spans="1:28" ht="15" customHeight="1">
-      <c r="A256" s="67"/>
+      <c r="A256" s="55"/>
       <c r="B256" s="3">
         <v>46366</v>
       </c>
@@ -17530,7 +17542,7 @@
       <c r="AB256" s="4"/>
     </row>
     <row r="257" spans="1:28" ht="15" customHeight="1">
-      <c r="A257" s="67"/>
+      <c r="A257" s="55"/>
       <c r="B257" s="3">
         <v>46367</v>
       </c>
@@ -17562,7 +17574,7 @@
       <c r="AB257" s="4"/>
     </row>
     <row r="258" spans="1:28" ht="15" customHeight="1">
-      <c r="A258" s="67"/>
+      <c r="A258" s="55"/>
       <c r="B258" s="3">
         <v>46368</v>
       </c>
@@ -17594,7 +17606,7 @@
       <c r="AB258" s="4"/>
     </row>
     <row r="259" spans="1:28" ht="15" customHeight="1">
-      <c r="A259" s="67"/>
+      <c r="A259" s="55"/>
       <c r="B259" s="3">
         <v>46369</v>
       </c>
@@ -17626,7 +17638,7 @@
       <c r="AB259" s="4"/>
     </row>
     <row r="260" spans="1:28" ht="15" customHeight="1">
-      <c r="A260" s="67"/>
+      <c r="A260" s="55"/>
       <c r="B260" s="3">
         <v>46370</v>
       </c>
@@ -17658,7 +17670,7 @@
       <c r="AB260" s="4"/>
     </row>
     <row r="261" spans="1:28" ht="15" customHeight="1">
-      <c r="A261" s="67"/>
+      <c r="A261" s="55"/>
       <c r="B261" s="3">
         <v>46371</v>
       </c>
@@ -17690,7 +17702,7 @@
       <c r="AB261" s="4"/>
     </row>
     <row r="262" spans="1:28" ht="15" customHeight="1">
-      <c r="A262" s="67"/>
+      <c r="A262" s="55"/>
       <c r="B262" s="3">
         <v>46372</v>
       </c>
@@ -17722,7 +17734,7 @@
       <c r="AB262" s="4"/>
     </row>
     <row r="263" spans="1:28" ht="15" customHeight="1">
-      <c r="A263" s="67"/>
+      <c r="A263" s="55"/>
       <c r="B263" s="3">
         <v>46373</v>
       </c>
@@ -17754,7 +17766,7 @@
       <c r="AB263" s="4"/>
     </row>
     <row r="264" spans="1:28" ht="15" customHeight="1">
-      <c r="A264" s="67"/>
+      <c r="A264" s="55"/>
       <c r="B264" s="3">
         <v>46374</v>
       </c>
@@ -17786,7 +17798,7 @@
       <c r="AB264" s="4"/>
     </row>
     <row r="265" spans="1:28" ht="15" customHeight="1">
-      <c r="A265" s="67"/>
+      <c r="A265" s="55"/>
       <c r="B265" s="3">
         <v>46375</v>
       </c>
@@ -17818,7 +17830,7 @@
       <c r="AB265" s="4"/>
     </row>
     <row r="266" spans="1:28" ht="15" customHeight="1">
-      <c r="A266" s="67"/>
+      <c r="A266" s="55"/>
       <c r="B266" s="3">
         <v>46376</v>
       </c>
@@ -17850,7 +17862,7 @@
       <c r="AB266" s="4"/>
     </row>
     <row r="267" spans="1:28" ht="15" customHeight="1">
-      <c r="A267" s="67"/>
+      <c r="A267" s="55"/>
       <c r="B267" s="3">
         <v>46377</v>
       </c>
@@ -17882,7 +17894,7 @@
       <c r="AB267" s="4"/>
     </row>
     <row r="268" spans="1:28" ht="15" customHeight="1">
-      <c r="A268" s="67"/>
+      <c r="A268" s="55"/>
       <c r="B268" s="3">
         <v>46378</v>
       </c>
@@ -17914,7 +17926,7 @@
       <c r="AB268" s="4"/>
     </row>
     <row r="269" spans="1:28" ht="15" customHeight="1">
-      <c r="A269" s="67"/>
+      <c r="A269" s="55"/>
       <c r="B269" s="3">
         <v>46379</v>
       </c>
@@ -17946,7 +17958,7 @@
       <c r="AB269" s="4"/>
     </row>
     <row r="270" spans="1:28" ht="15" customHeight="1">
-      <c r="A270" s="67"/>
+      <c r="A270" s="55"/>
       <c r="B270" s="3">
         <v>46380</v>
       </c>
@@ -17978,7 +17990,7 @@
       <c r="AB270" s="4"/>
     </row>
     <row r="271" spans="1:28" ht="15" customHeight="1">
-      <c r="A271" s="67"/>
+      <c r="A271" s="55"/>
       <c r="B271" s="3">
         <v>46381</v>
       </c>
@@ -18010,7 +18022,7 @@
       <c r="AB271" s="4"/>
     </row>
     <row r="272" spans="1:28" ht="15" customHeight="1">
-      <c r="A272" s="67"/>
+      <c r="A272" s="55"/>
       <c r="B272" s="3">
         <v>46382</v>
       </c>
@@ -18042,7 +18054,7 @@
       <c r="AB272" s="4"/>
     </row>
     <row r="273" spans="1:28" ht="15" customHeight="1">
-      <c r="A273" s="67"/>
+      <c r="A273" s="55"/>
       <c r="B273" s="3">
         <v>46383</v>
       </c>
@@ -18074,7 +18086,7 @@
       <c r="AB273" s="4"/>
     </row>
     <row r="274" spans="1:28" ht="15" customHeight="1">
-      <c r="A274" s="67"/>
+      <c r="A274" s="55"/>
       <c r="B274" s="3">
         <v>46384</v>
       </c>
@@ -18106,7 +18118,7 @@
       <c r="AB274" s="4"/>
     </row>
     <row r="275" spans="1:28" ht="15" customHeight="1">
-      <c r="A275" s="67"/>
+      <c r="A275" s="55"/>
       <c r="B275" s="3">
         <v>46385</v>
       </c>
@@ -18138,7 +18150,7 @@
       <c r="AB275" s="4"/>
     </row>
     <row r="276" spans="1:28" ht="15.75" customHeight="1">
-      <c r="A276" s="67"/>
+      <c r="A276" s="55"/>
       <c r="B276" s="3">
         <v>46386</v>
       </c>
@@ -18170,7 +18182,7 @@
       <c r="AB276" s="4"/>
     </row>
     <row r="277" spans="1:28" ht="15.75" thickBot="1">
-      <c r="A277" s="67"/>
+      <c r="A277" s="55"/>
       <c r="B277" s="3">
         <v>46387</v>
       </c>
@@ -18202,7 +18214,7 @@
       <c r="AB277" s="4"/>
     </row>
     <row r="278" spans="1:28" ht="27" customHeight="1">
-      <c r="A278" s="66" t="s">
+      <c r="A278" s="54" t="s">
         <v>37</v>
       </c>
       <c r="B278" s="7">
@@ -18236,7 +18248,7 @@
       <c r="AB278" s="8"/>
     </row>
     <row r="279" spans="1:28">
-      <c r="A279" s="67"/>
+      <c r="A279" s="55"/>
       <c r="B279" s="3">
         <v>46389</v>
       </c>
@@ -18268,7 +18280,7 @@
       <c r="AB279" s="4"/>
     </row>
     <row r="280" spans="1:28">
-      <c r="A280" s="67"/>
+      <c r="A280" s="55"/>
       <c r="B280" s="3">
         <v>46390</v>
       </c>
@@ -18300,7 +18312,7 @@
       <c r="AB280" s="4"/>
     </row>
     <row r="281" spans="1:28">
-      <c r="A281" s="67"/>
+      <c r="A281" s="55"/>
       <c r="B281" s="3">
         <v>46391</v>
       </c>
@@ -18332,7 +18344,7 @@
       <c r="AB281" s="4"/>
     </row>
     <row r="282" spans="1:28">
-      <c r="A282" s="67"/>
+      <c r="A282" s="55"/>
       <c r="B282" s="3">
         <v>46392</v>
       </c>
@@ -18364,7 +18376,7 @@
       <c r="AB282" s="4"/>
     </row>
     <row r="283" spans="1:28">
-      <c r="A283" s="67"/>
+      <c r="A283" s="55"/>
       <c r="B283" s="3">
         <v>46393</v>
       </c>
@@ -18396,7 +18408,7 @@
       <c r="AB283" s="4"/>
     </row>
     <row r="284" spans="1:28">
-      <c r="A284" s="67"/>
+      <c r="A284" s="55"/>
       <c r="B284" s="3">
         <v>46394</v>
       </c>
@@ -18428,7 +18440,7 @@
       <c r="AB284" s="4"/>
     </row>
     <row r="285" spans="1:28">
-      <c r="A285" s="67"/>
+      <c r="A285" s="55"/>
       <c r="B285" s="3">
         <v>46395</v>
       </c>
@@ -18460,7 +18472,7 @@
       <c r="AB285" s="4"/>
     </row>
     <row r="286" spans="1:28">
-      <c r="A286" s="67"/>
+      <c r="A286" s="55"/>
       <c r="B286" s="3">
         <v>46396</v>
       </c>
@@ -18492,7 +18504,7 @@
       <c r="AB286" s="4"/>
     </row>
     <row r="287" spans="1:28">
-      <c r="A287" s="67"/>
+      <c r="A287" s="55"/>
       <c r="B287" s="3">
         <v>46397</v>
       </c>
@@ -18524,7 +18536,7 @@
       <c r="AB287" s="4"/>
     </row>
     <row r="288" spans="1:28">
-      <c r="A288" s="67"/>
+      <c r="A288" s="55"/>
       <c r="B288" s="3">
         <v>46398</v>
       </c>
@@ -18556,7 +18568,7 @@
       <c r="AB288" s="4"/>
     </row>
     <row r="289" spans="1:28">
-      <c r="A289" s="67"/>
+      <c r="A289" s="55"/>
       <c r="B289" s="3">
         <v>46399</v>
       </c>
@@ -18588,7 +18600,7 @@
       <c r="AB289" s="4"/>
     </row>
     <row r="290" spans="1:28">
-      <c r="A290" s="67"/>
+      <c r="A290" s="55"/>
       <c r="B290" s="3">
         <v>46400</v>
       </c>
@@ -18620,7 +18632,7 @@
       <c r="AB290" s="4"/>
     </row>
     <row r="291" spans="1:28">
-      <c r="A291" s="67"/>
+      <c r="A291" s="55"/>
       <c r="B291" s="3">
         <v>46401</v>
       </c>
@@ -18652,7 +18664,7 @@
       <c r="AB291" s="4"/>
     </row>
     <row r="292" spans="1:28">
-      <c r="A292" s="67"/>
+      <c r="A292" s="55"/>
       <c r="B292" s="3">
         <v>46402</v>
       </c>
@@ -18684,7 +18696,7 @@
       <c r="AB292" s="4"/>
     </row>
     <row r="293" spans="1:28">
-      <c r="A293" s="67"/>
+      <c r="A293" s="55"/>
       <c r="B293" s="3">
         <v>46403</v>
       </c>
@@ -18716,7 +18728,7 @@
       <c r="AB293" s="4"/>
     </row>
     <row r="294" spans="1:28">
-      <c r="A294" s="67"/>
+      <c r="A294" s="55"/>
       <c r="B294" s="3">
         <v>46404</v>
       </c>
@@ -18748,7 +18760,7 @@
       <c r="AB294" s="4"/>
     </row>
     <row r="295" spans="1:28">
-      <c r="A295" s="67"/>
+      <c r="A295" s="55"/>
       <c r="B295" s="3">
         <v>46405</v>
       </c>
@@ -18780,7 +18792,7 @@
       <c r="AB295" s="4"/>
     </row>
     <row r="296" spans="1:28">
-      <c r="A296" s="67"/>
+      <c r="A296" s="55"/>
       <c r="B296" s="3">
         <v>46406</v>
       </c>
@@ -18812,7 +18824,7 @@
       <c r="AB296" s="4"/>
     </row>
     <row r="297" spans="1:28">
-      <c r="A297" s="67"/>
+      <c r="A297" s="55"/>
       <c r="B297" s="3">
         <v>46407</v>
       </c>
@@ -18844,7 +18856,7 @@
       <c r="AB297" s="4"/>
     </row>
     <row r="298" spans="1:28">
-      <c r="A298" s="67"/>
+      <c r="A298" s="55"/>
       <c r="B298" s="3">
         <v>46408</v>
       </c>
@@ -18876,7 +18888,7 @@
       <c r="AB298" s="4"/>
     </row>
     <row r="299" spans="1:28">
-      <c r="A299" s="67"/>
+      <c r="A299" s="55"/>
       <c r="B299" s="3">
         <v>46409</v>
       </c>
@@ -18908,7 +18920,7 @@
       <c r="AB299" s="4"/>
     </row>
     <row r="300" spans="1:28">
-      <c r="A300" s="67"/>
+      <c r="A300" s="55"/>
       <c r="B300" s="3">
         <v>46410</v>
       </c>
@@ -18940,7 +18952,7 @@
       <c r="AB300" s="4"/>
     </row>
     <row r="301" spans="1:28">
-      <c r="A301" s="67"/>
+      <c r="A301" s="55"/>
       <c r="B301" s="3">
         <v>46411</v>
       </c>
@@ -18972,7 +18984,7 @@
       <c r="AB301" s="4"/>
     </row>
     <row r="302" spans="1:28">
-      <c r="A302" s="67"/>
+      <c r="A302" s="55"/>
       <c r="B302" s="3">
         <v>46412</v>
       </c>
@@ -19004,7 +19016,7 @@
       <c r="AB302" s="4"/>
     </row>
     <row r="303" spans="1:28">
-      <c r="A303" s="67"/>
+      <c r="A303" s="55"/>
       <c r="B303" s="3">
         <v>46413</v>
       </c>
@@ -19036,7 +19048,7 @@
       <c r="AB303" s="4"/>
     </row>
     <row r="304" spans="1:28">
-      <c r="A304" s="67"/>
+      <c r="A304" s="55"/>
       <c r="B304" s="3">
         <v>46414</v>
       </c>
@@ -19068,7 +19080,7 @@
       <c r="AB304" s="4"/>
     </row>
     <row r="305" spans="1:28">
-      <c r="A305" s="67"/>
+      <c r="A305" s="55"/>
       <c r="B305" s="3">
         <v>46415</v>
       </c>
@@ -19100,7 +19112,7 @@
       <c r="AB305" s="4"/>
     </row>
     <row r="306" spans="1:28">
-      <c r="A306" s="67"/>
+      <c r="A306" s="55"/>
       <c r="B306" s="3">
         <v>46416</v>
       </c>
@@ -19132,7 +19144,7 @@
       <c r="AB306" s="4"/>
     </row>
     <row r="307" spans="1:28">
-      <c r="A307" s="67"/>
+      <c r="A307" s="55"/>
       <c r="B307" s="3">
         <v>46417</v>
       </c>
@@ -19164,7 +19176,7 @@
       <c r="AB307" s="4"/>
     </row>
     <row r="308" spans="1:28" ht="15.75" thickBot="1">
-      <c r="A308" s="67"/>
+      <c r="A308" s="55"/>
       <c r="B308" s="3">
         <v>46418</v>
       </c>
@@ -19196,7 +19208,7 @@
       <c r="AB308" s="4"/>
     </row>
     <row r="309" spans="1:28">
-      <c r="A309" s="66" t="s">
+      <c r="A309" s="54" t="s">
         <v>38</v>
       </c>
       <c r="B309" s="7">
@@ -19230,7 +19242,7 @@
       <c r="AB309" s="8"/>
     </row>
     <row r="310" spans="1:28">
-      <c r="A310" s="67"/>
+      <c r="A310" s="55"/>
       <c r="B310" s="3">
         <v>46420</v>
       </c>
@@ -19262,7 +19274,7 @@
       <c r="AB310" s="4"/>
     </row>
     <row r="311" spans="1:28">
-      <c r="A311" s="67"/>
+      <c r="A311" s="55"/>
       <c r="B311" s="3">
         <v>46421</v>
       </c>
@@ -19294,7 +19306,7 @@
       <c r="AB311" s="4"/>
     </row>
     <row r="312" spans="1:28">
-      <c r="A312" s="67"/>
+      <c r="A312" s="55"/>
       <c r="B312" s="3">
         <v>46422</v>
       </c>
@@ -19326,7 +19338,7 @@
       <c r="AB312" s="4"/>
     </row>
     <row r="313" spans="1:28">
-      <c r="A313" s="67"/>
+      <c r="A313" s="55"/>
       <c r="B313" s="3">
         <v>46423</v>
       </c>
@@ -19358,7 +19370,7 @@
       <c r="AB313" s="4"/>
     </row>
     <row r="314" spans="1:28">
-      <c r="A314" s="67"/>
+      <c r="A314" s="55"/>
       <c r="B314" s="3">
         <v>46424</v>
       </c>
@@ -19390,7 +19402,7 @@
       <c r="AB314" s="4"/>
     </row>
     <row r="315" spans="1:28">
-      <c r="A315" s="67"/>
+      <c r="A315" s="55"/>
       <c r="B315" s="3">
         <v>46425</v>
       </c>
@@ -19422,7 +19434,7 @@
       <c r="AB315" s="4"/>
     </row>
     <row r="316" spans="1:28">
-      <c r="A316" s="67"/>
+      <c r="A316" s="55"/>
       <c r="B316" s="3">
         <v>46426</v>
       </c>
@@ -19454,7 +19466,7 @@
       <c r="AB316" s="4"/>
     </row>
     <row r="317" spans="1:28">
-      <c r="A317" s="67"/>
+      <c r="A317" s="55"/>
       <c r="B317" s="3">
         <v>46427</v>
       </c>
@@ -19486,7 +19498,7 @@
       <c r="AB317" s="4"/>
     </row>
     <row r="318" spans="1:28">
-      <c r="A318" s="67"/>
+      <c r="A318" s="55"/>
       <c r="B318" s="3">
         <v>46428</v>
       </c>
@@ -19518,7 +19530,7 @@
       <c r="AB318" s="4"/>
     </row>
     <row r="319" spans="1:28">
-      <c r="A319" s="67"/>
+      <c r="A319" s="55"/>
       <c r="B319" s="3">
         <v>46429</v>
       </c>
@@ -19550,7 +19562,7 @@
       <c r="AB319" s="4"/>
     </row>
     <row r="320" spans="1:28">
-      <c r="A320" s="67"/>
+      <c r="A320" s="55"/>
       <c r="B320" s="3">
         <v>46430</v>
       </c>
@@ -19582,7 +19594,7 @@
       <c r="AB320" s="4"/>
     </row>
     <row r="321" spans="1:28">
-      <c r="A321" s="67"/>
+      <c r="A321" s="55"/>
       <c r="B321" s="3">
         <v>46431</v>
       </c>
@@ -19614,7 +19626,7 @@
       <c r="AB321" s="4"/>
     </row>
     <row r="322" spans="1:28">
-      <c r="A322" s="67"/>
+      <c r="A322" s="55"/>
       <c r="B322" s="3">
         <v>46432</v>
       </c>
@@ -19646,7 +19658,7 @@
       <c r="AB322" s="4"/>
     </row>
     <row r="323" spans="1:28">
-      <c r="A323" s="67"/>
+      <c r="A323" s="55"/>
       <c r="B323" s="3">
         <v>46433</v>
       </c>
@@ -19678,7 +19690,7 @@
       <c r="AB323" s="4"/>
     </row>
     <row r="324" spans="1:28">
-      <c r="A324" s="67"/>
+      <c r="A324" s="55"/>
       <c r="B324" s="3">
         <v>46434</v>
       </c>
@@ -19710,7 +19722,7 @@
       <c r="AB324" s="4"/>
     </row>
     <row r="325" spans="1:28">
-      <c r="A325" s="67"/>
+      <c r="A325" s="55"/>
       <c r="B325" s="3">
         <v>46435</v>
       </c>
@@ -19742,7 +19754,7 @@
       <c r="AB325" s="4"/>
     </row>
     <row r="326" spans="1:28">
-      <c r="A326" s="67"/>
+      <c r="A326" s="55"/>
       <c r="B326" s="3">
         <v>46436</v>
       </c>
@@ -19774,7 +19786,7 @@
       <c r="AB326" s="4"/>
     </row>
     <row r="327" spans="1:28">
-      <c r="A327" s="67"/>
+      <c r="A327" s="55"/>
       <c r="B327" s="3">
         <v>46437</v>
       </c>
@@ -19806,7 +19818,7 @@
       <c r="AB327" s="4"/>
     </row>
     <row r="328" spans="1:28">
-      <c r="A328" s="67"/>
+      <c r="A328" s="55"/>
       <c r="B328" s="3">
         <v>46438</v>
       </c>
@@ -19838,7 +19850,7 @@
       <c r="AB328" s="4"/>
     </row>
     <row r="329" spans="1:28">
-      <c r="A329" s="67"/>
+      <c r="A329" s="55"/>
       <c r="B329" s="3">
         <v>46439</v>
       </c>
@@ -19870,7 +19882,7 @@
       <c r="AB329" s="4"/>
     </row>
     <row r="330" spans="1:28">
-      <c r="A330" s="67"/>
+      <c r="A330" s="55"/>
       <c r="B330" s="3">
         <v>46440</v>
       </c>
@@ -19902,7 +19914,7 @@
       <c r="AB330" s="4"/>
     </row>
     <row r="331" spans="1:28">
-      <c r="A331" s="67"/>
+      <c r="A331" s="55"/>
       <c r="B331" s="3">
         <v>46441</v>
       </c>
@@ -19934,7 +19946,7 @@
       <c r="AB331" s="4"/>
     </row>
     <row r="332" spans="1:28">
-      <c r="A332" s="67"/>
+      <c r="A332" s="55"/>
       <c r="B332" s="3">
         <v>46442</v>
       </c>
@@ -19966,7 +19978,7 @@
       <c r="AB332" s="4"/>
     </row>
     <row r="333" spans="1:28">
-      <c r="A333" s="67"/>
+      <c r="A333" s="55"/>
       <c r="B333" s="3">
         <v>46443</v>
       </c>
@@ -19998,7 +20010,7 @@
       <c r="AB333" s="4"/>
     </row>
     <row r="334" spans="1:28">
-      <c r="A334" s="67"/>
+      <c r="A334" s="55"/>
       <c r="B334" s="3">
         <v>46444</v>
       </c>
@@ -20030,7 +20042,7 @@
       <c r="AB334" s="4"/>
     </row>
     <row r="335" spans="1:28">
-      <c r="A335" s="67"/>
+      <c r="A335" s="55"/>
       <c r="B335" s="3">
         <v>46445</v>
       </c>
@@ -20062,7 +20074,7 @@
       <c r="AB335" s="4"/>
     </row>
     <row r="336" spans="1:28" ht="15.75" thickBot="1">
-      <c r="A336" s="67"/>
+      <c r="A336" s="55"/>
       <c r="B336" s="3">
         <v>46446</v>
       </c>
@@ -20094,7 +20106,7 @@
       <c r="AB336" s="4"/>
     </row>
     <row r="337" spans="1:28">
-      <c r="A337" s="66" t="s">
+      <c r="A337" s="54" t="s">
         <v>39</v>
       </c>
       <c r="B337" s="7">
@@ -20128,7 +20140,7 @@
       <c r="AB337" s="8"/>
     </row>
     <row r="338" spans="1:28">
-      <c r="A338" s="67"/>
+      <c r="A338" s="55"/>
       <c r="B338" s="3">
         <v>46448</v>
       </c>
@@ -20160,7 +20172,7 @@
       <c r="AB338" s="4"/>
     </row>
     <row r="339" spans="1:28">
-      <c r="A339" s="67"/>
+      <c r="A339" s="55"/>
       <c r="B339" s="3">
         <v>46449</v>
       </c>
@@ -20192,7 +20204,7 @@
       <c r="AB339" s="4"/>
     </row>
     <row r="340" spans="1:28">
-      <c r="A340" s="67"/>
+      <c r="A340" s="55"/>
       <c r="B340" s="3">
         <v>46450</v>
       </c>
@@ -20224,7 +20236,7 @@
       <c r="AB340" s="4"/>
     </row>
     <row r="341" spans="1:28">
-      <c r="A341" s="67"/>
+      <c r="A341" s="55"/>
       <c r="B341" s="3">
         <v>46451</v>
       </c>
@@ -20256,7 +20268,7 @@
       <c r="AB341" s="4"/>
     </row>
     <row r="342" spans="1:28">
-      <c r="A342" s="67"/>
+      <c r="A342" s="55"/>
       <c r="B342" s="3">
         <v>46452</v>
       </c>
@@ -20288,7 +20300,7 @@
       <c r="AB342" s="4"/>
     </row>
     <row r="343" spans="1:28">
-      <c r="A343" s="67"/>
+      <c r="A343" s="55"/>
       <c r="B343" s="3">
         <v>46453</v>
       </c>
@@ -20320,7 +20332,7 @@
       <c r="AB343" s="4"/>
     </row>
     <row r="344" spans="1:28">
-      <c r="A344" s="67"/>
+      <c r="A344" s="55"/>
       <c r="B344" s="3">
         <v>46454</v>
       </c>
@@ -20352,7 +20364,7 @@
       <c r="AB344" s="4"/>
     </row>
     <row r="345" spans="1:28">
-      <c r="A345" s="67"/>
+      <c r="A345" s="55"/>
       <c r="B345" s="3">
         <v>46455</v>
       </c>
@@ -20384,7 +20396,7 @@
       <c r="AB345" s="4"/>
     </row>
     <row r="346" spans="1:28">
-      <c r="A346" s="67"/>
+      <c r="A346" s="55"/>
       <c r="B346" s="3">
         <v>46456</v>
       </c>
@@ -20416,7 +20428,7 @@
       <c r="AB346" s="4"/>
     </row>
     <row r="347" spans="1:28">
-      <c r="A347" s="67"/>
+      <c r="A347" s="55"/>
       <c r="B347" s="3">
         <v>46457</v>
       </c>
@@ -20448,7 +20460,7 @@
       <c r="AB347" s="4"/>
     </row>
     <row r="348" spans="1:28">
-      <c r="A348" s="67"/>
+      <c r="A348" s="55"/>
       <c r="B348" s="3">
         <v>46458</v>
       </c>
@@ -20480,7 +20492,7 @@
       <c r="AB348" s="4"/>
     </row>
     <row r="349" spans="1:28">
-      <c r="A349" s="67"/>
+      <c r="A349" s="55"/>
       <c r="B349" s="3">
         <v>46459</v>
       </c>
@@ -20512,7 +20524,7 @@
       <c r="AB349" s="4"/>
     </row>
     <row r="350" spans="1:28">
-      <c r="A350" s="67"/>
+      <c r="A350" s="55"/>
       <c r="B350" s="3">
         <v>46460</v>
       </c>
@@ -20544,7 +20556,7 @@
       <c r="AB350" s="4"/>
     </row>
     <row r="351" spans="1:28">
-      <c r="A351" s="67"/>
+      <c r="A351" s="55"/>
       <c r="B351" s="3">
         <v>46461</v>
       </c>
@@ -20576,7 +20588,7 @@
       <c r="AB351" s="4"/>
     </row>
     <row r="352" spans="1:28">
-      <c r="A352" s="67"/>
+      <c r="A352" s="55"/>
       <c r="B352" s="3">
         <v>46462</v>
       </c>
@@ -20608,7 +20620,7 @@
       <c r="AB352" s="4"/>
     </row>
     <row r="353" spans="1:28">
-      <c r="A353" s="67"/>
+      <c r="A353" s="55"/>
       <c r="B353" s="3">
         <v>46463</v>
       </c>
@@ -20640,7 +20652,7 @@
       <c r="AB353" s="4"/>
     </row>
     <row r="354" spans="1:28">
-      <c r="A354" s="67"/>
+      <c r="A354" s="55"/>
       <c r="B354" s="3">
         <v>46464</v>
       </c>
@@ -20672,7 +20684,7 @@
       <c r="AB354" s="4"/>
     </row>
     <row r="355" spans="1:28">
-      <c r="A355" s="67"/>
+      <c r="A355" s="55"/>
       <c r="B355" s="3">
         <v>46465</v>
       </c>
@@ -20704,7 +20716,7 @@
       <c r="AB355" s="4"/>
     </row>
     <row r="356" spans="1:28">
-      <c r="A356" s="67"/>
+      <c r="A356" s="55"/>
       <c r="B356" s="3">
         <v>46466</v>
       </c>
@@ -20736,7 +20748,7 @@
       <c r="AB356" s="4"/>
     </row>
     <row r="357" spans="1:28">
-      <c r="A357" s="67"/>
+      <c r="A357" s="55"/>
       <c r="B357" s="3">
         <v>46467</v>
       </c>
@@ -20768,7 +20780,7 @@
       <c r="AB357" s="4"/>
     </row>
     <row r="358" spans="1:28">
-      <c r="A358" s="67"/>
+      <c r="A358" s="55"/>
       <c r="B358" s="3">
         <v>46468</v>
       </c>
@@ -20800,7 +20812,7 @@
       <c r="AB358" s="4"/>
     </row>
     <row r="359" spans="1:28">
-      <c r="A359" s="67"/>
+      <c r="A359" s="55"/>
       <c r="B359" s="3">
         <v>46469</v>
       </c>
@@ -20832,7 +20844,7 @@
       <c r="AB359" s="4"/>
     </row>
     <row r="360" spans="1:28">
-      <c r="A360" s="67"/>
+      <c r="A360" s="55"/>
       <c r="B360" s="3">
         <v>46470</v>
       </c>
@@ -20864,7 +20876,7 @@
       <c r="AB360" s="4"/>
     </row>
     <row r="361" spans="1:28">
-      <c r="A361" s="67"/>
+      <c r="A361" s="55"/>
       <c r="B361" s="3">
         <v>46471</v>
       </c>
@@ -20896,7 +20908,7 @@
       <c r="AB361" s="4"/>
     </row>
     <row r="362" spans="1:28">
-      <c r="A362" s="67"/>
+      <c r="A362" s="55"/>
       <c r="B362" s="3">
         <v>46472</v>
       </c>
@@ -20928,7 +20940,7 @@
       <c r="AB362" s="4"/>
     </row>
     <row r="363" spans="1:28">
-      <c r="A363" s="67"/>
+      <c r="A363" s="55"/>
       <c r="B363" s="3">
         <v>46473</v>
       </c>
@@ -20960,7 +20972,7 @@
       <c r="AB363" s="4"/>
     </row>
     <row r="364" spans="1:28" ht="15.75" thickBot="1">
-      <c r="A364" s="67"/>
+      <c r="A364" s="55"/>
       <c r="B364" s="3">
         <v>46474</v>
       </c>
@@ -20992,7 +21004,7 @@
       <c r="AB364" s="4"/>
     </row>
     <row r="365" spans="1:28">
-      <c r="A365" s="66"/>
+      <c r="A365" s="54"/>
       <c r="B365" s="3">
         <v>46475</v>
       </c>
@@ -21024,7 +21036,7 @@
       <c r="AB365" s="4"/>
     </row>
     <row r="366" spans="1:28">
-      <c r="A366" s="67"/>
+      <c r="A366" s="55"/>
       <c r="B366" s="3">
         <v>46476</v>
       </c>
@@ -21056,7 +21068,7 @@
       <c r="AB366" s="4"/>
     </row>
     <row r="367" spans="1:28">
-      <c r="A367" s="67"/>
+      <c r="A367" s="55"/>
       <c r="B367" s="3">
         <v>46477</v>
       </c>
@@ -21089,13 +21101,11 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="A278:A308"/>
-    <mergeCell ref="A309:A336"/>
-    <mergeCell ref="A337:A364"/>
-    <mergeCell ref="A365:A367"/>
-    <mergeCell ref="A186:A216"/>
-    <mergeCell ref="A217:A246"/>
-    <mergeCell ref="A247:A277"/>
+    <mergeCell ref="A64:A93"/>
+    <mergeCell ref="A94:A124"/>
+    <mergeCell ref="A125:A155"/>
+    <mergeCell ref="A156:A185"/>
+    <mergeCell ref="A33:A63"/>
     <mergeCell ref="U1:AB1"/>
     <mergeCell ref="O1:Q1"/>
     <mergeCell ref="R1:T1"/>
@@ -21106,18 +21116,20 @@
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="I1:K1"/>
     <mergeCell ref="L1:N1"/>
-    <mergeCell ref="A64:A93"/>
-    <mergeCell ref="A94:A124"/>
-    <mergeCell ref="A125:A155"/>
-    <mergeCell ref="A156:A185"/>
-    <mergeCell ref="A33:A63"/>
+    <mergeCell ref="A278:A308"/>
+    <mergeCell ref="A309:A336"/>
+    <mergeCell ref="A337:A364"/>
+    <mergeCell ref="A365:A367"/>
+    <mergeCell ref="A186:A216"/>
+    <mergeCell ref="A217:A246"/>
+    <mergeCell ref="A247:A277"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation type="decimal" operator="greaterThanOrEqual" showErrorMessage="1" error="Enter a number ≥ 0" sqref="X3:Z185 U204:V367 L3:T367 X204:Z367">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="decimal" showErrorMessage="1" errorTitle="Hours" error="Enter hours between 0 and 24 (19.5 = 19 h 30 min)" sqref="AB204:AB367 F3:H367 I3:I196 J3:K185 I202:K367 AA3:AA367 AB3:AB185">
+    <dataValidation type="decimal" showErrorMessage="1" errorTitle="Hours" error="Enter hours between 0 and 24 (19.5 = 19 h 30 min)" sqref="AB204:AB367 I3:I196 J3:K185 AB3:AB185 AA3:AA367 I202:K367 F3:H367">
       <formula1>0</formula1>
       <formula2>24</formula2>
     </dataValidation>
@@ -26021,74 +26033,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="21">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="49" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="74" t="s">
+      <c r="B1" s="52" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="20.25">
-      <c r="A2" s="72" t="s">
+      <c r="A2" s="50" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="75">
+      <c r="B2" s="53">
         <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="20.25">
-      <c r="A3" s="72" t="s">
+      <c r="A3" s="50" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="75">
+      <c r="B3" s="53">
         <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="20.25">
-      <c r="A4" s="72" t="s">
-        <v>24</v>
-      </c>
-      <c r="B4" s="75">
+      <c r="A4" s="50" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="53">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="20.25">
-      <c r="A5" s="72" t="s">
+      <c r="A5" s="50" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="75">
+      <c r="B5" s="53">
         <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="20.25">
-      <c r="A6" s="72" t="s">
+      <c r="A6" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="75">
+      <c r="B6" s="53">
         <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="20.25">
-      <c r="A7" s="72" t="s">
+      <c r="A7" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="75">
+      <c r="B7" s="53">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="20.25">
-      <c r="A8" s="72" t="s">
+      <c r="A8" s="50" t="s">
         <v>42</v>
       </c>
-      <c r="B8" s="75">
+      <c r="B8" s="53">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="20.25">
-      <c r="A9" s="71" t="s">
+      <c r="A9" s="49" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="73">
+      <c r="B9" s="51">
         <f>SUM(B2:B8)</f>
         <v>139</v>
       </c>

</xml_diff>